<commit_message>
More re-org, add debug mode, effectiveness
</commit_message>
<xml_diff>
--- a/legacy/vivarium_gates_lsff_by_wealth_quintile/0100_data_prep/extraction/Data Extraction Sheet.xlsx
+++ b/legacy/vivarium_gates_lsff_by_wealth_quintile/0100_data_prep/extraction/Data Extraction Sheet.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27927"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27930"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uwnetid.sharepoint.com/sites/ihme_simulation_science_team/Shared Documents/Research/LSFF/04_Concept_Model_Development/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CC6D7F9C-56D5-4A5D-BAA4-9192B6B9B393}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F48EAE2D-6B6A-4FFF-A505-D5D23FEECF86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" firstSheet="3" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Country-Vehicle Progress" sheetId="1" r:id="rId1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1509" uniqueCount="214">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1550" uniqueCount="216">
   <si>
     <t>Country</t>
   </si>
@@ -320,6 +320,9 @@
   </si>
   <si>
     <t>N/A</t>
+  </si>
+  <si>
+    <t>Baseline effective % of fortified</t>
   </si>
   <si>
     <t>concentration</t>
@@ -346,6 +349,9 @@
   </si>
   <si>
     <t>Originally in mcg/100g; https://www.wolframalpha.com/input?i=4.25+mg+per+100+grams+in+micrograms+per+gram</t>
+  </si>
+  <si>
+    <t>Same as intervention, for now</t>
   </si>
   <si>
     <t>Pregnant people hemoglobin levels at baseline</t>
@@ -642,7 +648,7 @@
     <t>Intervention coverage % of fortifiable and unfortified</t>
   </si>
   <si>
-    <t>Intervention effective % of newly fortified</t>
+    <t>Intervention effective % of fortified</t>
   </si>
   <si>
     <t>Andy Garcia email 7/26</t>
@@ -927,7 +933,17 @@
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="13">
+  <dxfs count="14">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -1610,7 +1626,7 @@
     <mergeCell ref="F2:G2"/>
   </mergeCells>
   <conditionalFormatting sqref="B5:G9">
-    <cfRule type="cellIs" dxfId="12" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="13" priority="1" operator="equal">
       <formula>"Missing"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -1686,25 +1702,25 @@
     </row>
     <row r="4" spans="1:7">
       <c r="A4" s="30" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="B4" s="31" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="C4" s="31" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="D4" s="31" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="E4" s="31" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="F4" s="31" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="G4" s="31" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
     </row>
     <row r="5" spans="1:7">
@@ -1718,7 +1734,7 @@
     </row>
     <row r="6" spans="1:7">
       <c r="A6" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B6" t="str">
         <f>IF(COUNTIFS('Scenario Definition Extraction'!$A$2:$A$991, B$1,  'Scenario Definition Extraction'!$B$2:$B$991, B$2,  'Scenario Definition Extraction'!$C$2:$C$991, B$3, 'Scenario Definition Extraction'!$D$2:$D$991, B$4, 'Scenario Definition Extraction'!$E$2:$E$991, $A6) = 0, "Missing", "Complete")</f>
@@ -1747,7 +1763,7 @@
     </row>
     <row r="7" spans="1:7">
       <c r="A7" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="B7" t="str">
         <f>IF(COUNTIFS('Scenario Definition Extraction'!$A$2:$A$991, B$1,  'Scenario Definition Extraction'!$B$2:$B$991, B$2,  'Scenario Definition Extraction'!$C$2:$C$991, B$3, 'Scenario Definition Extraction'!$D$2:$D$991, B$4, 'Scenario Definition Extraction'!$E$2:$E$991, $A7) = 0, "Missing", "Complete")</f>
@@ -1776,7 +1792,7 @@
     </row>
     <row r="8" spans="1:7">
       <c r="A8" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B8" t="str">
         <f>IF(COUNTIFS('Scenario Definition Extraction'!$A$2:$A$991, B$1,  'Scenario Definition Extraction'!$B$2:$B$991, B$2,  'Scenario Definition Extraction'!$C$2:$C$991, B$3, 'Scenario Definition Extraction'!$D$2:$D$991, B$4, 'Scenario Definition Extraction'!$E$2:$E$991, $A8) = 0, "Missing", "Complete")</f>
@@ -1887,7 +1903,7 @@
         <v>83</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>11</v>
@@ -1919,10 +1935,10 @@
         <v>85</v>
       </c>
       <c r="D2" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="E2" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="F2" t="s">
         <v>29</v>
@@ -1931,13 +1947,13 @@
         <v>30</v>
       </c>
       <c r="H2" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="I2" s="7">
         <v>0.8</v>
       </c>
       <c r="J2" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -1951,10 +1967,10 @@
         <v>84</v>
       </c>
       <c r="D3" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="E3" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="F3" t="s">
         <v>29</v>
@@ -1963,13 +1979,13 @@
         <v>30</v>
       </c>
       <c r="H3" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="I3" s="7">
         <v>0.8</v>
       </c>
       <c r="J3" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -1983,10 +1999,10 @@
         <v>84</v>
       </c>
       <c r="D4" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="E4" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="F4" t="s">
         <v>29</v>
@@ -1995,13 +2011,13 @@
         <v>30</v>
       </c>
       <c r="H4" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="I4" s="7">
         <v>0.8</v>
       </c>
       <c r="J4" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
     </row>
     <row r="5" spans="1:10">
@@ -2015,10 +2031,10 @@
         <v>84</v>
       </c>
       <c r="D5" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="E5" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="F5" t="s">
         <v>29</v>
@@ -2027,13 +2043,13 @@
         <v>30</v>
       </c>
       <c r="H5" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="I5" s="7">
         <v>0.8</v>
       </c>
       <c r="J5" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
     </row>
     <row r="6" spans="1:10">
@@ -2047,10 +2063,10 @@
         <v>85</v>
       </c>
       <c r="D6" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="E6" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="F6" t="s">
         <v>29</v>
@@ -2059,13 +2075,13 @@
         <v>30</v>
       </c>
       <c r="H6" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="I6" s="7">
         <v>0.8</v>
       </c>
       <c r="J6" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
     </row>
     <row r="7" spans="1:10">
@@ -2079,10 +2095,10 @@
         <v>84</v>
       </c>
       <c r="D7" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="E7" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="F7" t="s">
         <v>29</v>
@@ -2091,13 +2107,13 @@
         <v>30</v>
       </c>
       <c r="H7" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="I7" s="7">
         <v>0.8</v>
       </c>
       <c r="J7" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
     </row>
     <row r="8" spans="1:10">
@@ -2111,10 +2127,10 @@
         <v>85</v>
       </c>
       <c r="D8" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="E8" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="F8" t="s">
         <v>29</v>
@@ -2123,13 +2139,13 @@
         <v>30</v>
       </c>
       <c r="H8" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="I8" s="7">
         <v>0.8</v>
       </c>
       <c r="J8" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
     </row>
     <row r="9" spans="1:10">
@@ -2143,10 +2159,10 @@
         <v>84</v>
       </c>
       <c r="D9" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="E9" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="F9" t="s">
         <v>29</v>
@@ -2155,13 +2171,13 @@
         <v>30</v>
       </c>
       <c r="H9" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="I9" s="7">
         <v>0.8</v>
       </c>
       <c r="J9" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
     </row>
     <row r="10" spans="1:10">
@@ -2175,10 +2191,10 @@
         <v>84</v>
       </c>
       <c r="D10" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="E10" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="F10" t="s">
         <v>29</v>
@@ -2187,13 +2203,13 @@
         <v>30</v>
       </c>
       <c r="H10" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="I10" s="7">
         <v>0.8</v>
       </c>
       <c r="J10" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
     </row>
     <row r="11" spans="1:10">
@@ -2207,10 +2223,10 @@
         <v>84</v>
       </c>
       <c r="D11" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="E11" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="F11" t="s">
         <v>29</v>
@@ -2219,13 +2235,13 @@
         <v>30</v>
       </c>
       <c r="H11" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="I11" s="7">
         <v>0.8</v>
       </c>
       <c r="J11" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
     </row>
     <row r="12" spans="1:10">
@@ -2239,10 +2255,10 @@
         <v>85</v>
       </c>
       <c r="D12" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="E12" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="F12" t="s">
         <v>29</v>
@@ -2251,13 +2267,13 @@
         <v>30</v>
       </c>
       <c r="H12" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="I12" s="7">
         <v>0.8</v>
       </c>
       <c r="J12" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
     </row>
     <row r="13" spans="1:10">
@@ -2271,10 +2287,10 @@
         <v>84</v>
       </c>
       <c r="D13" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="E13" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="F13" t="s">
         <v>29</v>
@@ -2283,13 +2299,13 @@
         <v>30</v>
       </c>
       <c r="H13" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="I13" s="7">
         <v>0.8</v>
       </c>
       <c r="J13" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
     </row>
     <row r="14" spans="1:10">
@@ -2303,25 +2319,25 @@
         <v>85</v>
       </c>
       <c r="D14" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="E14" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="F14" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="G14" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="H14" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="I14">
         <v>840</v>
       </c>
       <c r="J14" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
     </row>
     <row r="15" spans="1:10">
@@ -2335,25 +2351,25 @@
         <v>84</v>
       </c>
       <c r="D15" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="E15" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="F15" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="G15" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="H15" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="I15">
         <v>24</v>
       </c>
       <c r="J15" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
     </row>
     <row r="16" spans="1:10">
@@ -2367,25 +2383,25 @@
         <v>84</v>
       </c>
       <c r="D16" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="E16" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="F16" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="G16" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="H16" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="I16">
         <v>14.084507042253522</v>
       </c>
       <c r="J16" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
     </row>
     <row r="17" spans="1:10">
@@ -2399,25 +2415,25 @@
         <v>84</v>
       </c>
       <c r="D17" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="E17" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="F17" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="G17" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="H17" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="I17">
         <v>56.338028169014088</v>
       </c>
       <c r="J17" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
     </row>
     <row r="18" spans="1:10">
@@ -2431,25 +2447,25 @@
         <v>85</v>
       </c>
       <c r="D18" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="E18" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="F18" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="G18" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="H18" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="I18">
         <v>42.5</v>
       </c>
       <c r="J18" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
     </row>
     <row r="19" spans="1:10">
@@ -2463,25 +2479,25 @@
         <v>84</v>
       </c>
       <c r="D19" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="E19" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="F19" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="G19" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="H19" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="I19">
         <v>0.125</v>
       </c>
       <c r="J19" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
     </row>
   </sheetData>
@@ -2531,22 +2547,22 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>21</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="45">
@@ -2554,13 +2570,13 @@
         <v>49</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="C2" s="6" t="s">
         <v>51</v>
       </c>
       <c r="D2" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="E2">
         <v>2021</v>
@@ -2568,30 +2584,30 @@
     </row>
     <row r="3" spans="1:6">
       <c r="A3" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B3" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="B4" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="D4" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="E4" s="16" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="F4" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
     </row>
   </sheetData>
@@ -4904,7 +4920,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0EC50408-61D8-4A10-93E8-9867356C2F54}">
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:M8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="52.42578125" bestFit="1" customWidth="1"/>
@@ -5065,11 +5081,11 @@
         <v>87</v>
       </c>
       <c r="H6" t="str">
-        <f>IF(COUNTIFS('Country-Vehicle-Fort Extraction'!$A$2:$A$938, F$1,  'Country-Vehicle-Fort Extraction'!$B$2:$B$938, F$2,  'Country-Vehicle-Fort Extraction'!$C$2:$C$938, H$3, 'Country-Vehicle-Fort Extraction'!$D$2:$D$938, "All",  'Country-Vehicle-Fort Extraction'!$E$2:$E$938, $A6, 'Country-Vehicle-Fort Extraction'!$J$2:$J$938, "&lt;&gt;") = 0, "Missing", "Complete")</f>
-        <v>Missing</v>
+        <f>IF(COUNTIFS('Country-Vehicle-Fort Extraction'!$A$2:$A$940, F$1,  'Country-Vehicle-Fort Extraction'!$B$2:$B$940, F$2,  'Country-Vehicle-Fort Extraction'!$C$2:$C$940, H$3, 'Country-Vehicle-Fort Extraction'!$D$2:$D$940, "Total",  'Country-Vehicle-Fort Extraction'!$E$2:$E$940, $A6, 'Country-Vehicle-Fort Extraction'!$J$2:$J$940, "&lt;&gt;") = 0, "Missing", "Complete")</f>
+        <v>Complete</v>
       </c>
       <c r="I6" t="str">
-        <f>IF(COUNTIFS('Country-Vehicle-Fort Extraction'!$A$2:$A$938, F$1,  'Country-Vehicle-Fort Extraction'!$B$2:$B$938, F$2,  'Country-Vehicle-Fort Extraction'!$C$2:$C$938, H$3, 'Country-Vehicle-Fort Extraction'!$D$2:$D$938, "&lt;&gt;All",  'Country-Vehicle-Fort Extraction'!$E$2:$E$938, $A6, 'Country-Vehicle-Fort Extraction'!$J$2:$J$938, "&lt;&gt;") &lt; 5, "Missing", "Complete")</f>
+        <f>IF(COUNTIFS('Country-Vehicle-Fort Extraction'!$A$2:$A$940, F$1,  'Country-Vehicle-Fort Extraction'!$B$2:$B$940, F$2,  'Country-Vehicle-Fort Extraction'!$C$2:$C$940, H$3, 'Country-Vehicle-Fort Extraction'!$D$2:$D$940, "&lt;&gt;All",  'Country-Vehicle-Fort Extraction'!$E$2:$E$940, $A6, 'Country-Vehicle-Fort Extraction'!$J$2:$J$940, "&lt;&gt;") &lt; 5, "Missing", "Complete")</f>
         <v>Complete</v>
       </c>
       <c r="J6" t="s">
@@ -5108,25 +5124,70 @@
         <v>87</v>
       </c>
       <c r="H7" t="str">
-        <f>IF(COUNTIFS('Country-Vehicle-Fort Extraction'!$A$2:$A$938, F$1,  'Country-Vehicle-Fort Extraction'!$B$2:$B$938, F$2,  'Country-Vehicle-Fort Extraction'!$C$2:$C$938, H$3, 'Country-Vehicle-Fort Extraction'!$D$2:$D$938, "All",  'Country-Vehicle-Fort Extraction'!$E$2:$E$938, $A7, 'Country-Vehicle-Fort Extraction'!$J$2:$J$938, "&lt;&gt;") = 0, "Missing", "Complete")</f>
+        <f>IF(COUNTIFS('Country-Vehicle-Fort Extraction'!$A$2:$A$940, F$1,  'Country-Vehicle-Fort Extraction'!$B$2:$B$940, F$2,  'Country-Vehicle-Fort Extraction'!$C$2:$C$940, H$3, 'Country-Vehicle-Fort Extraction'!$D$2:$D$940, "Total",  'Country-Vehicle-Fort Extraction'!$E$2:$E$940, $A7, 'Country-Vehicle-Fort Extraction'!$J$2:$J$940, "&lt;&gt;") = 0, "Missing", "Complete")</f>
         <v>Missing</v>
       </c>
       <c r="I7" t="str">
-        <f>IF(COUNTIFS('Country-Vehicle-Fort Extraction'!$A$2:$A$938, F$1,  'Country-Vehicle-Fort Extraction'!$B$2:$B$938, F$2,  'Country-Vehicle-Fort Extraction'!$C$2:$C$938, H$3, 'Country-Vehicle-Fort Extraction'!$D$2:$D$938, "&lt;&gt;All",  'Country-Vehicle-Fort Extraction'!$E$2:$E$938, $A7, 'Country-Vehicle-Fort Extraction'!$J$2:$J$938, "&lt;&gt;") &lt; 5, "Missing", "Complete")</f>
+        <f>IF(COUNTIFS('Country-Vehicle-Fort Extraction'!$A$2:$A$940, F$1,  'Country-Vehicle-Fort Extraction'!$B$2:$B$940, F$2,  'Country-Vehicle-Fort Extraction'!$C$2:$C$940, H$3, 'Country-Vehicle-Fort Extraction'!$D$2:$D$940, "&lt;&gt;Total",  'Country-Vehicle-Fort Extraction'!$E$2:$E$940, $A7, 'Country-Vehicle-Fort Extraction'!$J$2:$J$940, "&lt;&gt;") &lt; 5, "Missing", "Complete")</f>
         <v>Missing</v>
       </c>
       <c r="J7" t="str">
-        <f>IF(COUNTIFS('Country-Vehicle-Fort Extraction'!$A$2:$A$938, J$1,  'Country-Vehicle-Fort Extraction'!$B$2:$B$938, J$2,  'Country-Vehicle-Fort Extraction'!$C$2:$C$938, J$3, 'Country-Vehicle-Fort Extraction'!$D$2:$D$938, "All",  'Country-Vehicle-Fort Extraction'!$E$2:$E$938, $A7, 'Country-Vehicle-Fort Extraction'!$J$2:$J$938, "&lt;&gt;") = 0, "Missing", "Complete")</f>
+        <f>IF(COUNTIFS('Country-Vehicle-Fort Extraction'!$A$2:$A$940, J$1,  'Country-Vehicle-Fort Extraction'!$B$2:$B$940, J$2,  'Country-Vehicle-Fort Extraction'!$C$2:$C$940, J$3, 'Country-Vehicle-Fort Extraction'!$D$2:$D$940, "All",  'Country-Vehicle-Fort Extraction'!$E$2:$E$940, $A7, 'Country-Vehicle-Fort Extraction'!$J$2:$J$940, "&lt;&gt;") = 0, "Missing", "Complete")</f>
         <v>Missing</v>
       </c>
       <c r="K7" t="s">
         <v>90</v>
       </c>
       <c r="L7" t="str">
-        <f>IF(COUNTIFS('Country-Vehicle-Fort Extraction'!$A$2:$A$938, J$1,  'Country-Vehicle-Fort Extraction'!$B$2:$B$938, J$2,  'Country-Vehicle-Fort Extraction'!$C$2:$C$938, L$3, 'Country-Vehicle-Fort Extraction'!$D$2:$D$938, "All",  'Country-Vehicle-Fort Extraction'!$E$2:$E$938, $A7, 'Country-Vehicle-Fort Extraction'!$J$2:$J$938, "&lt;&gt;") = 0, "Missing", "Complete")</f>
+        <f>IF(COUNTIFS('Country-Vehicle-Fort Extraction'!$A$2:$A$940, J$1,  'Country-Vehicle-Fort Extraction'!$B$2:$B$940, J$2,  'Country-Vehicle-Fort Extraction'!$C$2:$C$940, L$3, 'Country-Vehicle-Fort Extraction'!$D$2:$D$940, "All",  'Country-Vehicle-Fort Extraction'!$E$2:$E$940, $A7, 'Country-Vehicle-Fort Extraction'!$J$2:$J$940, "&lt;&gt;") = 0, "Missing", "Complete")</f>
         <v>Missing</v>
       </c>
       <c r="M7" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13">
+      <c r="A8" t="s">
+        <v>91</v>
+      </c>
+      <c r="B8" t="s">
+        <v>87</v>
+      </c>
+      <c r="C8" t="s">
+        <v>87</v>
+      </c>
+      <c r="D8" t="s">
+        <v>88</v>
+      </c>
+      <c r="E8" t="s">
+        <v>88</v>
+      </c>
+      <c r="F8" t="s">
+        <v>87</v>
+      </c>
+      <c r="G8" t="s">
+        <v>87</v>
+      </c>
+      <c r="H8" t="str">
+        <f>IF(COUNTIFS('Country-Vehicle-Fort Extraction'!$A$2:$A$940, F$1,  'Country-Vehicle-Fort Extraction'!$B$2:$B$940, F$2,  'Country-Vehicle-Fort Extraction'!$C$2:$C$940, H$3, 'Country-Vehicle-Fort Extraction'!$D$2:$D$940, "Total",  'Country-Vehicle-Fort Extraction'!$E$2:$E$940, $A8, 'Country-Vehicle-Fort Extraction'!$J$2:$J$940, "&lt;&gt;") = 0, "Missing", "Complete")</f>
+        <v>Missing</v>
+      </c>
+      <c r="I8" t="str">
+        <f>IF(COUNTIFS('Country-Vehicle-Fort Extraction'!$A$2:$A$940, F$1,  'Country-Vehicle-Fort Extraction'!$B$2:$B$940, F$2,  'Country-Vehicle-Fort Extraction'!$C$2:$C$940, H$3, 'Country-Vehicle-Fort Extraction'!$D$2:$D$940, "&lt;&gt;Total",  'Country-Vehicle-Fort Extraction'!$E$2:$E$940, $A8, 'Country-Vehicle-Fort Extraction'!$J$2:$J$940, "&lt;&gt;") &lt; 5, "Missing", "Complete")</f>
+        <v>Missing</v>
+      </c>
+      <c r="J8" t="str">
+        <f>IF(COUNTIFS('Country-Vehicle-Fort Extraction'!$A$2:$A$940, J$1,  'Country-Vehicle-Fort Extraction'!$B$2:$B$940, J$2,  'Country-Vehicle-Fort Extraction'!$C$2:$C$940, J$3, 'Country-Vehicle-Fort Extraction'!$D$2:$D$940, "All",  'Country-Vehicle-Fort Extraction'!$E$2:$E$940, $A8, 'Country-Vehicle-Fort Extraction'!$J$2:$J$940, "&lt;&gt;") = 0, "Missing", "Complete")</f>
+        <v>Missing</v>
+      </c>
+      <c r="K8" t="s">
+        <v>90</v>
+      </c>
+      <c r="L8" t="str">
+        <f>IF(COUNTIFS('Country-Vehicle-Fort Extraction'!$A$2:$A$940, J$1,  'Country-Vehicle-Fort Extraction'!$B$2:$B$940, J$2,  'Country-Vehicle-Fort Extraction'!$C$2:$C$940, L$3, 'Country-Vehicle-Fort Extraction'!$D$2:$D$940, "All",  'Country-Vehicle-Fort Extraction'!$E$2:$E$940, $A8, 'Country-Vehicle-Fort Extraction'!$J$2:$J$940, "&lt;&gt;") = 0, "Missing", "Complete")</f>
+        <v>Missing</v>
+      </c>
+      <c r="M8" t="s">
         <v>90</v>
       </c>
     </row>
@@ -5146,7 +5207,12 @@
     <mergeCell ref="H3:I3"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:M6 B7:I7 I6:M7">
-    <cfRule type="cellIs" dxfId="11" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="12" priority="7" operator="equal">
+      <formula>"Missing"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H8:M8">
+    <cfRule type="cellIs" dxfId="11" priority="1" operator="equal">
       <formula>"Missing"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5156,7 +5222,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC26D125-533B-4E2C-8B10-83B96EF6CBCB}">
-  <dimension ref="A1:L14"/>
+  <dimension ref="A1:L18"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="8" bestFit="1" customWidth="1"/>
@@ -5252,10 +5318,10 @@
         <v>89</v>
       </c>
       <c r="F3" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="I3" t="s">
         <v>47</v>
@@ -5293,7 +5359,7 @@
         <v>0.61875637104994907</v>
       </c>
       <c r="L4" s="9" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="5" spans="1:12">
@@ -5463,10 +5529,10 @@
         <v>89</v>
       </c>
       <c r="F10" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="G10" s="8" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="I10" t="s">
         <v>47</v>
@@ -5475,7 +5541,7 @@
         <v>650</v>
       </c>
       <c r="L10" s="9" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="11" spans="1:12">
@@ -5507,7 +5573,7 @@
         <v>0</v>
       </c>
       <c r="L11" s="9" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
     </row>
     <row r="12" spans="1:12">
@@ -5527,10 +5593,10 @@
         <v>89</v>
       </c>
       <c r="F12" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="G12" s="8" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="I12" t="s">
         <v>47</v>
@@ -5540,7 +5606,7 @@
       </c>
       <c r="L12" s="9"/>
     </row>
-    <row r="13" spans="1:12">
+    <row r="13" spans="1:12" ht="43.5">
       <c r="A13" t="s">
         <v>3</v>
       </c>
@@ -5557,19 +5623,19 @@
         <v>89</v>
       </c>
       <c r="F13" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="G13" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="I13" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="J13">
         <v>42.5</v>
       </c>
-      <c r="L13" t="s">
-        <v>97</v>
+      <c r="L13" s="5" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="14" spans="1:12">
@@ -5589,19 +5655,135 @@
         <v>89</v>
       </c>
       <c r="F14" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="G14" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="I14" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="J14">
         <v>0.125</v>
       </c>
       <c r="L14" s="9" t="s">
-        <v>98</v>
+        <v>99</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12">
+      <c r="A15" t="s">
+        <v>2</v>
+      </c>
+      <c r="B15" t="s">
+        <v>6</v>
+      </c>
+      <c r="C15" t="s">
+        <v>85</v>
+      </c>
+      <c r="D15" t="s">
+        <v>27</v>
+      </c>
+      <c r="E15" t="s">
+        <v>91</v>
+      </c>
+      <c r="F15" t="s">
+        <v>29</v>
+      </c>
+      <c r="G15" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="J15" s="7">
+        <v>0.8</v>
+      </c>
+      <c r="L15" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12">
+      <c r="A16" t="s">
+        <v>2</v>
+      </c>
+      <c r="B16" t="s">
+        <v>6</v>
+      </c>
+      <c r="C16" t="s">
+        <v>84</v>
+      </c>
+      <c r="D16" t="s">
+        <v>27</v>
+      </c>
+      <c r="E16" t="s">
+        <v>91</v>
+      </c>
+      <c r="F16" t="s">
+        <v>29</v>
+      </c>
+      <c r="G16" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="J16" s="7">
+        <v>0.8</v>
+      </c>
+      <c r="L16" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12">
+      <c r="A17" t="s">
+        <v>3</v>
+      </c>
+      <c r="B17" t="s">
+        <v>7</v>
+      </c>
+      <c r="C17" t="s">
+        <v>85</v>
+      </c>
+      <c r="D17" t="s">
+        <v>27</v>
+      </c>
+      <c r="E17" t="s">
+        <v>91</v>
+      </c>
+      <c r="F17" t="s">
+        <v>29</v>
+      </c>
+      <c r="G17" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="J17" s="7">
+        <v>0.8</v>
+      </c>
+      <c r="L17" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12">
+      <c r="A18" t="s">
+        <v>3</v>
+      </c>
+      <c r="B18" t="s">
+        <v>7</v>
+      </c>
+      <c r="C18" t="s">
+        <v>84</v>
+      </c>
+      <c r="D18" t="s">
+        <v>27</v>
+      </c>
+      <c r="E18" t="s">
+        <v>91</v>
+      </c>
+      <c r="F18" t="s">
+        <v>29</v>
+      </c>
+      <c r="G18" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="J18" s="7">
+        <v>0.8</v>
+      </c>
+      <c r="L18" t="s">
+        <v>100</v>
       </c>
     </row>
   </sheetData>
@@ -5701,7 +5883,7 @@
     </row>
     <row r="4" spans="1:8">
       <c r="A4" s="4" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B4" t="s">
         <v>88</v>
@@ -5710,21 +5892,21 @@
         <v>88</v>
       </c>
       <c r="D4" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="E4" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="F4" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="G4" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
     </row>
     <row r="5" spans="1:8">
       <c r="A5" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B5" t="str">
         <f>IF(COUNTIFS('Country Extraction'!$A$2:$A$980, B$1,  'Country Extraction'!$B$2:$B$980, "All",  'Country Extraction'!$C$2:$C$980, $A5) = 0, "Missing", "Complete")</f>
@@ -5753,7 +5935,7 @@
     </row>
     <row r="6" spans="1:8">
       <c r="A6" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B6" t="str">
         <f>IF(COUNTIFS('Country Extraction'!$A$2:$A$980, B$1,  'Country Extraction'!$B$2:$B$980, "All",  'Country Extraction'!$C$2:$C$980, $A6) = 0, "Missing", "Complete")</f>
@@ -5782,7 +5964,7 @@
     </row>
     <row r="7" spans="1:8">
       <c r="A7" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B7" t="s">
         <v>88</v>
@@ -5791,21 +5973,21 @@
         <v>88</v>
       </c>
       <c r="D7" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="E7" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="F7" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="G7" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
     </row>
     <row r="8" spans="1:8">
       <c r="A8" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B8" t="s">
         <v>88</v>
@@ -5814,21 +5996,21 @@
         <v>88</v>
       </c>
       <c r="D8" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="E8" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="F8" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="G8" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
     </row>
     <row r="9" spans="1:8">
       <c r="A9" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B9" t="s">
         <v>88</v>
@@ -5837,24 +6019,24 @@
         <v>88</v>
       </c>
       <c r="D9" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="E9" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="F9" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="G9" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="H9" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
     <row r="10" spans="1:8">
       <c r="A10" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B10" t="s">
         <v>88</v>
@@ -5863,26 +6045,26 @@
         <v>88</v>
       </c>
       <c r="D10" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="E10" t="str">
         <f>IF(COUNTIFS('Country Extraction'!$A$1:$A$995, F$1, 'Country Extraction'!$B$1:$B$995, "&lt;&gt;All", 'Country Extraction'!$C$1:$C$995, $A10, 'Country Extraction'!$H$1:$H$995, "&lt;&gt;") &lt; 5, "Missing", "Complete")</f>
         <v>Missing</v>
       </c>
       <c r="F10" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="G10" t="str">
         <f>IF(COUNTIFS('Country Extraction'!$A$1:$A$995, H$1, 'Country Extraction'!$B$1:$B$995, "&lt;&gt;All", 'Country Extraction'!$C$1:$C$995, $A10, 'Country Extraction'!$H$1:$H$995, "&lt;&gt;") &lt; 5, "Missing", "Complete")</f>
         <v>Missing</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
     <row r="11" spans="1:8">
       <c r="A11" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B11" t="s">
         <v>88</v>
@@ -5891,25 +6073,25 @@
         <v>88</v>
       </c>
       <c r="D11" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="E11" t="str">
         <f>IF(COUNTIFS('Country Extraction'!$A$1:$A$995, F$1, 'Country Extraction'!$B$1:$B$995, "&lt;&gt;All", 'Country Extraction'!$C$1:$C$995, $A11, 'Country Extraction'!$H$1:$H$995, "&lt;&gt;") &lt; 5, "Missing", "Complete")</f>
         <v>Missing</v>
       </c>
       <c r="F11" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="G11" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="H11" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
     </row>
     <row r="12" spans="1:8">
       <c r="A12" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B12" t="s">
         <v>88</v>
@@ -5918,21 +6100,21 @@
         <v>88</v>
       </c>
       <c r="D12" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="E12" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="F12" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="G12" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
     </row>
     <row r="13" spans="1:8">
       <c r="A13" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B13" t="s">
         <v>88</v>
@@ -5941,24 +6123,24 @@
         <v>88</v>
       </c>
       <c r="D13" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="E13" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="F13" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="G13" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="H13" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
     </row>
     <row r="14" spans="1:8">
       <c r="A14" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B14" t="s">
         <v>88</v>
@@ -5967,41 +6149,41 @@
         <v>88</v>
       </c>
       <c r="D14" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="E14" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="F14" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="G14" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="H14" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
     </row>
     <row r="15" spans="1:8">
       <c r="A15" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B15" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="C15" t="str">
         <f>IF(COUNTIFS('Country Extraction'!$A$1:$A$995, D$1, 'Country Extraction'!$B$1:$B$995, "&lt;&gt;All", 'Country Extraction'!$C$1:$C$995, $A15, 'Country Extraction'!$H$1:$H$995, "&lt;&gt;") &lt; 5, "Missing", "Complete")</f>
         <v>Missing</v>
       </c>
       <c r="D15" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="E15" t="str">
         <f>IF(COUNTIFS('Country Extraction'!$A$1:$A$995, F$1, 'Country Extraction'!$B$1:$B$995, "&lt;&gt;All", 'Country Extraction'!$C$1:$C$995, $A15, 'Country Extraction'!$H$1:$H$995, "&lt;&gt;") &lt; 5, "Missing", "Complete")</f>
         <v>Missing</v>
       </c>
       <c r="F15" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="G15" t="str">
         <f>IF(COUNTIFS('Country Extraction'!$A$1:$A$995, H$1, 'Country Extraction'!$B$1:$B$995, "&lt;&gt;All", 'Country Extraction'!$C$1:$C$995, $A15, 'Country Extraction'!$H$1:$H$995, "&lt;&gt;") &lt; 5, "Missing", "Complete")</f>
@@ -6072,19 +6254,19 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="E2" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="G2" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="J2" s="11" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="32.25" customHeight="1">
@@ -6095,16 +6277,16 @@
         <v>37</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="E3" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="G3" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="J3" s="13" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -6115,13 +6297,13 @@
         <v>38</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="E4" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="G4" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="5" spans="1:10">
@@ -6132,13 +6314,13 @@
         <v>39</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="E5" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="G5" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="6" spans="1:10">
@@ -6149,13 +6331,13 @@
         <v>40</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="E6" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="G6" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="7" spans="1:10">
@@ -6166,115 +6348,115 @@
         <v>41</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="E7" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="G7" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="8" spans="1:10">
       <c r="A8" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B8" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="E8" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="G8" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="9" spans="1:10">
       <c r="A9" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B9" t="s">
         <v>37</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="E9" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="G9" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="10" spans="1:10">
       <c r="A10" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B10" t="s">
         <v>38</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="E10" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="G10" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="11" spans="1:10">
       <c r="A11" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B11" t="s">
         <v>39</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="E11" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="G11" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="12" spans="1:10">
       <c r="A12" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B12" t="s">
         <v>40</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="E12" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="G12" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="13" spans="1:10">
       <c r="A13" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B13" t="s">
         <v>41</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="E13" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="G13" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="14" spans="1:10">
@@ -6282,16 +6464,16 @@
         <v>3</v>
       </c>
       <c r="B14" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C14" s="9" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="E14" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="G14" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="15" spans="1:10">
@@ -6302,13 +6484,13 @@
         <v>37</v>
       </c>
       <c r="C15" s="9" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="E15" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="G15" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="16" spans="1:10">
@@ -6319,13 +6501,13 @@
         <v>38</v>
       </c>
       <c r="C16" s="9" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="E16" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="G16" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="17" spans="1:10">
@@ -6336,13 +6518,13 @@
         <v>39</v>
       </c>
       <c r="C17" s="9" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="E17" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="G17" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="18" spans="1:10">
@@ -6353,13 +6535,13 @@
         <v>40</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="E18" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="G18" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="19" spans="1:10">
@@ -6370,13 +6552,13 @@
         <v>41</v>
       </c>
       <c r="C19" s="9" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="E19" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="G19" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="20" spans="1:10" ht="15.75">
@@ -6384,19 +6566,19 @@
         <v>1</v>
       </c>
       <c r="B20" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C20" s="9" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="E20" s="8" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="G20" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="J20" s="11" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
     </row>
     <row r="21" spans="1:10">
@@ -6407,16 +6589,16 @@
         <v>37</v>
       </c>
       <c r="C21" s="9" t="s">
+        <v>127</v>
+      </c>
+      <c r="E21" s="8" t="s">
+        <v>128</v>
+      </c>
+      <c r="G21" t="s">
+        <v>123</v>
+      </c>
+      <c r="J21" s="8" t="s">
         <v>125</v>
-      </c>
-      <c r="E21" s="8" t="s">
-        <v>126</v>
-      </c>
-      <c r="G21" t="s">
-        <v>121</v>
-      </c>
-      <c r="J21" s="8" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="22" spans="1:10">
@@ -6427,13 +6609,13 @@
         <v>38</v>
       </c>
       <c r="C22" s="9" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="E22" s="8" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="G22" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="23" spans="1:10">
@@ -6444,13 +6626,13 @@
         <v>39</v>
       </c>
       <c r="C23" s="9" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="E23" s="8" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="G23" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="24" spans="1:10">
@@ -6461,13 +6643,13 @@
         <v>40</v>
       </c>
       <c r="C24" s="9" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="E24" s="8" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="G24" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="25" spans="1:10">
@@ -6478,115 +6660,115 @@
         <v>41</v>
       </c>
       <c r="C25" s="9" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="E25" s="8" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="G25" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="26" spans="1:10">
       <c r="A26" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B26" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C26" s="9" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="E26" s="8" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="G26" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="27" spans="1:10">
       <c r="A27" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B27" t="s">
         <v>37</v>
       </c>
       <c r="C27" s="9" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="E27" s="8" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="G27" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="28" spans="1:10">
       <c r="A28" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B28" t="s">
         <v>38</v>
       </c>
       <c r="C28" s="9" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="E28" s="8" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="G28" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="29" spans="1:10">
       <c r="A29" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B29" t="s">
         <v>39</v>
       </c>
       <c r="C29" s="9" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="E29" s="8" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="G29" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="30" spans="1:10">
       <c r="A30" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B30" t="s">
         <v>40</v>
       </c>
       <c r="C30" s="9" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="E30" s="8" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="G30" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="31" spans="1:10">
       <c r="A31" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B31" t="s">
         <v>41</v>
       </c>
       <c r="C31" s="9" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="E31" s="8" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="G31" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="32" spans="1:10">
@@ -6594,16 +6776,16 @@
         <v>3</v>
       </c>
       <c r="B32" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C32" s="9" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="E32" s="8" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="G32" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="33" spans="1:7">
@@ -6614,13 +6796,13 @@
         <v>37</v>
       </c>
       <c r="C33" s="9" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="E33" s="8" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="G33" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="34" spans="1:7">
@@ -6631,13 +6813,13 @@
         <v>38</v>
       </c>
       <c r="C34" s="9" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="E34" s="8" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="G34" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="35" spans="1:7">
@@ -6648,13 +6830,13 @@
         <v>39</v>
       </c>
       <c r="C35" s="9" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="E35" s="8" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="G35" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="36" spans="1:7">
@@ -6665,13 +6847,13 @@
         <v>40</v>
       </c>
       <c r="C36" s="9" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="E36" s="8" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="G36" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="37" spans="1:7">
@@ -6682,13 +6864,13 @@
         <v>41</v>
       </c>
       <c r="C37" s="9" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="E37" s="8" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="G37" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="38" spans="1:7">
@@ -6696,13 +6878,13 @@
         <v>1</v>
       </c>
       <c r="B38" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C38" s="9" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="G38" s="9" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
     </row>
     <row r="39" spans="1:7">
@@ -6713,10 +6895,10 @@
         <v>37</v>
       </c>
       <c r="C39" s="9" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="G39" s="6" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
     <row r="40" spans="1:7">
@@ -6727,10 +6909,10 @@
         <v>38</v>
       </c>
       <c r="C40" s="9" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="G40" s="6" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
     <row r="41" spans="1:7">
@@ -6741,10 +6923,10 @@
         <v>39</v>
       </c>
       <c r="C41" s="9" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="G41" s="6" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
     <row r="42" spans="1:7">
@@ -6755,10 +6937,10 @@
         <v>40</v>
       </c>
       <c r="C42" s="9" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="G42" s="6" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
     <row r="43" spans="1:7">
@@ -6769,94 +6951,94 @@
         <v>41</v>
       </c>
       <c r="C43" s="9" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="G43" s="6" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
     <row r="44" spans="1:7">
       <c r="A44" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B44" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C44" s="9" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="G44" s="9" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
     </row>
     <row r="45" spans="1:7">
       <c r="A45" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B45" t="s">
         <v>37</v>
       </c>
       <c r="C45" s="9" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="G45" s="14" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
     </row>
     <row r="46" spans="1:7">
       <c r="A46" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B46" t="s">
         <v>38</v>
       </c>
       <c r="C46" s="9" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="G46" s="14" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
     </row>
     <row r="47" spans="1:7">
       <c r="A47" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B47" t="s">
         <v>39</v>
       </c>
       <c r="C47" s="9" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="G47" s="14" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
     </row>
     <row r="48" spans="1:7">
       <c r="A48" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B48" t="s">
         <v>40</v>
       </c>
       <c r="C48" s="9" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="G48" s="14" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
     </row>
     <row r="49" spans="1:10">
       <c r="A49" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B49" t="s">
         <v>41</v>
       </c>
       <c r="C49" s="9" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="G49" s="14" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
     </row>
     <row r="50" spans="1:10">
@@ -6864,13 +7046,13 @@
         <v>3</v>
       </c>
       <c r="B50" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C50" s="9" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="G50" s="9" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
     </row>
     <row r="51" spans="1:10">
@@ -6881,10 +7063,10 @@
         <v>37</v>
       </c>
       <c r="C51" s="9" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="G51" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="52" spans="1:10">
@@ -6895,10 +7077,10 @@
         <v>38</v>
       </c>
       <c r="C52" s="9" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="G52" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="53" spans="1:10">
@@ -6909,10 +7091,10 @@
         <v>39</v>
       </c>
       <c r="C53" s="9" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="G53" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="54" spans="1:10">
@@ -6923,10 +7105,10 @@
         <v>40</v>
       </c>
       <c r="C54" s="9" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="G54" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="55" spans="1:10">
@@ -6937,10 +7119,10 @@
         <v>41</v>
       </c>
       <c r="C55" s="9" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="G55" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="56" spans="1:10">
@@ -6948,13 +7130,13 @@
         <v>1</v>
       </c>
       <c r="B56" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C56" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G56" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
     </row>
     <row r="57" spans="1:10" ht="45">
@@ -6965,10 +7147,10 @@
         <v>37</v>
       </c>
       <c r="C57" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="J57" s="13" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
     </row>
     <row r="58" spans="1:10" ht="15.75">
@@ -6979,10 +7161,10 @@
         <v>38</v>
       </c>
       <c r="C58" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="J58" s="12" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
     </row>
     <row r="59" spans="1:10" ht="15.75">
@@ -6993,7 +7175,7 @@
         <v>39</v>
       </c>
       <c r="C59" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="J59" s="12"/>
     </row>
@@ -7005,7 +7187,7 @@
         <v>40</v>
       </c>
       <c r="C60" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
     </row>
     <row r="61" spans="1:10">
@@ -7016,76 +7198,76 @@
         <v>41</v>
       </c>
       <c r="C61" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
     </row>
     <row r="62" spans="1:10">
       <c r="A62" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B62" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C62" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G62" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
     </row>
     <row r="63" spans="1:10">
       <c r="A63" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B63" t="s">
         <v>37</v>
       </c>
       <c r="C63" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
     </row>
     <row r="64" spans="1:10">
       <c r="A64" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B64" t="s">
         <v>38</v>
       </c>
       <c r="C64" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
     </row>
     <row r="65" spans="1:10">
       <c r="A65" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B65" t="s">
         <v>39</v>
       </c>
       <c r="C65" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
     </row>
     <row r="66" spans="1:10">
       <c r="A66" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B66" t="s">
         <v>40</v>
       </c>
       <c r="C66" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
     </row>
     <row r="67" spans="1:10">
       <c r="A67" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B67" t="s">
         <v>41</v>
       </c>
       <c r="C67" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
     </row>
     <row r="68" spans="1:10">
@@ -7093,13 +7275,13 @@
         <v>3</v>
       </c>
       <c r="B68" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C68" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G68" s="15" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
     </row>
     <row r="69" spans="1:10">
@@ -7110,7 +7292,7 @@
         <v>37</v>
       </c>
       <c r="C69" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
     </row>
     <row r="70" spans="1:10">
@@ -7121,7 +7303,7 @@
         <v>38</v>
       </c>
       <c r="C70" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
     </row>
     <row r="71" spans="1:10">
@@ -7132,7 +7314,7 @@
         <v>39</v>
       </c>
       <c r="C71" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
     </row>
     <row r="72" spans="1:10">
@@ -7143,7 +7325,7 @@
         <v>40</v>
       </c>
       <c r="C72" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
     </row>
     <row r="73" spans="1:10">
@@ -7154,7 +7336,7 @@
         <v>41</v>
       </c>
       <c r="C73" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
     </row>
     <row r="74" spans="1:10" ht="30">
@@ -7162,36 +7344,36 @@
         <v>1</v>
       </c>
       <c r="B74" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C74" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="D74" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="G74" s="12" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="J74" s="14" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
     </row>
     <row r="75" spans="1:10">
       <c r="A75" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B75" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C75" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="D75" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="J75" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
     </row>
     <row r="76" spans="1:10">
@@ -7199,13 +7381,13 @@
         <v>3</v>
       </c>
       <c r="B76" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C76" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="D76" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
     </row>
   </sheetData>
@@ -7281,7 +7463,7 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="4" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B3" t="s">
         <v>88</v>
@@ -7297,7 +7479,7 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="26" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B4" t="s">
         <v>88</v>
@@ -7368,28 +7550,28 @@
         <v>7</v>
       </c>
       <c r="B2" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="C2" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="D2" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="E2" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="F2" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="G2" s="26">
         <v>3.25</v>
       </c>
       <c r="H2" s="26" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="I2" s="5" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
     </row>
     <row r="3" spans="1:9">
@@ -7397,28 +7579,28 @@
         <v>5</v>
       </c>
       <c r="B3" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="C3" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="D3" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="E3">
         <v>2021</v>
       </c>
       <c r="F3" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="G3">
         <v>4.4000000000000004</v>
       </c>
       <c r="H3" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="I3" s="6" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
     </row>
     <row r="4" spans="1:9">
@@ -7426,28 +7608,28 @@
         <v>6</v>
       </c>
       <c r="B4" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="C4" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="D4" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="E4">
         <v>2012</v>
       </c>
       <c r="F4" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="G4">
         <v>4.2</v>
       </c>
       <c r="H4" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="I4" s="6" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
     </row>
     <row r="5" spans="1:9">
@@ -7455,28 +7637,28 @@
         <v>7</v>
       </c>
       <c r="B5" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C5" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="D5" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="E5">
         <v>2013</v>
       </c>
       <c r="F5" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="G5">
         <v>16.7</v>
       </c>
       <c r="H5" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="I5" s="6" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
     </row>
     <row r="6" spans="1:9">
@@ -7484,28 +7666,28 @@
         <v>6</v>
       </c>
       <c r="B6" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C6" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="D6" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="E6">
         <v>2013</v>
       </c>
       <c r="F6" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="G6">
         <v>16.7</v>
       </c>
       <c r="H6" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="I6" s="6" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
     </row>
   </sheetData>
@@ -7577,7 +7759,7 @@
     </row>
     <row r="2" spans="1:9">
       <c r="A2" s="26" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B2" s="26"/>
       <c r="C2" s="26"/>
@@ -7590,59 +7772,59 @@
     </row>
     <row r="3" spans="1:9">
       <c r="A3" s="26" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B3" s="26" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="C3" s="26" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="D3" s="26">
         <v>2018</v>
       </c>
       <c r="E3" s="26" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="F3" s="26">
         <v>4.3</v>
       </c>
       <c r="G3" s="26" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="H3" s="24" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="I3" s="23"/>
     </row>
     <row r="4" spans="1:9">
       <c r="A4" s="26" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B4" s="26" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="C4" s="26" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="D4" s="26">
         <v>2015</v>
       </c>
       <c r="E4" s="25" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="F4" s="26">
         <v>6</v>
       </c>
       <c r="G4" s="27" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="H4" s="23"/>
       <c r="I4" s="23"/>
     </row>
     <row r="5" spans="1:9">
       <c r="A5" s="26" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B5" s="26"/>
       <c r="C5" s="26"/>
@@ -7655,18 +7837,18 @@
     </row>
     <row r="6" spans="1:9">
       <c r="A6" s="26" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B6" s="26" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="C6" s="26"/>
       <c r="D6" s="26"/>
       <c r="E6" s="26" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="F6" s="26" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="G6" s="26"/>
       <c r="H6" s="23"/>
@@ -7674,18 +7856,18 @@
     </row>
     <row r="7" spans="1:9">
       <c r="A7" s="26" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B7" s="26" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="C7" s="26"/>
       <c r="D7" s="26"/>
       <c r="E7" s="26" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="F7" s="26" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="G7" s="26"/>
       <c r="H7" s="23"/>
@@ -7693,22 +7875,22 @@
     </row>
     <row r="8" spans="1:9">
       <c r="A8" s="26" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="B8" s="26" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="C8" s="26"/>
       <c r="D8" s="26"/>
       <c r="E8" s="26" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="F8" s="26" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="G8" s="26"/>
       <c r="H8" s="23" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="I8" s="23"/>
     </row>
@@ -7787,6 +7969,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100447C4EFE3BCDC24F9D43FB479AF7E97A" ma:contentTypeVersion="17" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="710ccc9eba0c031f4d3c8297a7da4be2">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="19a3940c-c740-4699-845a-46837f99845a" xmlns:ns3="539a68f6-d0ac-4a73-9041-e1fa437c4cee" xmlns:ns4="ab06a5aa-8e31-4bdb-9b13-38c58a92ec8a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a67399e28ae6312d8947be2cafff42c1" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="19a3940c-c740-4699-845a-46837f99845a"/>
@@ -8040,7 +8231,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="ab06a5aa-8e31-4bdb-9b13-38c58a92ec8a" xsi:nil="true"/>
@@ -8051,23 +8242,14 @@
 </p:properties>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{44149C33-81B0-4C8D-A8B9-4C0F99EB683B}"/>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{302FEEF7-88D6-41D4-B999-EFF8511D95B1}"/>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4173999B-2FEB-4E5B-A6C7-6E33DD5EA2F7}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{44149C33-81B0-4C8D-A8B9-4C0F99EB683B}"/>
 </file>
</xml_diff>

<commit_message>
Incorporate folate models, generate first version of results spreadsheet
</commit_message>
<xml_diff>
--- a/legacy/vivarium_gates_lsff_by_wealth_quintile/0100_data_prep/extraction/Data Extraction Sheet.xlsx
+++ b/legacy/vivarium_gates_lsff_by_wealth_quintile/0100_data_prep/extraction/Data Extraction Sheet.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27930"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28004"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uwnetid.sharepoint.com/sites/ihme_simulation_science_team/Shared Documents/Research/LSFF/04_Concept_Model_Development/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F48EAE2D-6B6A-4FFF-A505-D5D23FEECF86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{B8CA6867-1011-45AB-BB75-EE63C249175B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" firstSheet="3" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1550" uniqueCount="216">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1558" uniqueCount="216">
   <si>
     <t>Country</t>
   </si>
@@ -5222,7 +5222,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC26D125-533B-4E2C-8B10-83B96EF6CBCB}">
-  <dimension ref="A1:L18"/>
+  <dimension ref="A1:L19"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="8" bestFit="1" customWidth="1"/>
@@ -5783,6 +5783,35 @@
         <v>0.8</v>
       </c>
       <c r="L18" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12">
+      <c r="A19" t="s">
+        <v>1</v>
+      </c>
+      <c r="B19" t="s">
+        <v>5</v>
+      </c>
+      <c r="C19" t="s">
+        <v>84</v>
+      </c>
+      <c r="D19" t="s">
+        <v>27</v>
+      </c>
+      <c r="E19" t="s">
+        <v>91</v>
+      </c>
+      <c r="F19" t="s">
+        <v>29</v>
+      </c>
+      <c r="G19" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="J19" s="7">
+        <v>0.8</v>
+      </c>
+      <c r="L19" t="s">
         <v>100</v>
       </c>
     </row>
@@ -7969,15 +7998,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100447C4EFE3BCDC24F9D43FB479AF7E97A" ma:contentTypeVersion="17" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="710ccc9eba0c031f4d3c8297a7da4be2">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="19a3940c-c740-4699-845a-46837f99845a" xmlns:ns3="539a68f6-d0ac-4a73-9041-e1fa437c4cee" xmlns:ns4="ab06a5aa-8e31-4bdb-9b13-38c58a92ec8a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a67399e28ae6312d8947be2cafff42c1" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="19a3940c-c740-4699-845a-46837f99845a"/>
@@ -8231,6 +8251,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -8243,11 +8272,11 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{44149C33-81B0-4C8D-A8B9-4C0F99EB683B}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{302FEEF7-88D6-41D4-B999-EFF8511D95B1}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{302FEEF7-88D6-41D4-B999-EFF8511D95B1}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{44149C33-81B0-4C8D-A8B9-4C0F99EB683B}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
Factor out hemoglobin, increase full-scale size, add example to non-pregnant anemia notebook, add cases to results spreadsheet
</commit_message>
<xml_diff>
--- a/legacy/vivarium_gates_lsff_by_wealth_quintile/0100_data_prep/extraction/Data Extraction Sheet.xlsx
+++ b/legacy/vivarium_gates_lsff_by_wealth_quintile/0100_data_prep/extraction/Data Extraction Sheet.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28004"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28005"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uwnetid.sharepoint.com/sites/ihme_simulation_science_team/Shared Documents/Research/LSFF/04_Concept_Model_Development/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B8CA6867-1011-45AB-BB75-EE63C249175B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{7934BE7B-3755-4AC0-B316-CDC44E903342}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" firstSheet="3" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -555,7 +555,7 @@
     <t>Anaemia, prenatal iron use, and risk of adverse pregnancy outcomes: systematic review and meta-analysis</t>
   </si>
   <si>
-    <t>7.29 to 26.11</t>
+    <t>0.729 to 2.611</t>
   </si>
   <si>
     <t>https://www.bmj.com/content/346/bmj.f3443; study of supplementation at higher doses than fortification; selected the effect among trials &lt;66mg/day as all fortification would fall in this range</t>
@@ -7542,6 +7542,7 @@
     <col min="3" max="3" width="19" customWidth="1"/>
     <col min="4" max="4" width="18.28515625" customWidth="1"/>
     <col min="6" max="6" width="34.140625" customWidth="1"/>
+    <col min="8" max="8" width="13.140625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="50.42578125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -7681,7 +7682,7 @@
         <v>160</v>
       </c>
       <c r="G5">
-        <v>16.7</v>
+        <v>1.67</v>
       </c>
       <c r="H5" t="s">
         <v>161</v>
@@ -7710,7 +7711,7 @@
         <v>160</v>
       </c>
       <c r="G6">
-        <v>16.7</v>
+        <v>1.67</v>
       </c>
       <c r="H6" t="s">
         <v>161</v>
@@ -7998,6 +7999,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="ab06a5aa-8e31-4bdb-9b13-38c58a92ec8a" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="19a3940c-c740-4699-845a-46837f99845a">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100447C4EFE3BCDC24F9D43FB479AF7E97A" ma:contentTypeVersion="17" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="710ccc9eba0c031f4d3c8297a7da4be2">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="19a3940c-c740-4699-845a-46837f99845a" xmlns:ns3="539a68f6-d0ac-4a73-9041-e1fa437c4cee" xmlns:ns4="ab06a5aa-8e31-4bdb-9b13-38c58a92ec8a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a67399e28ae6312d8947be2cafff42c1" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="19a3940c-c740-4699-845a-46837f99845a"/>
@@ -8251,28 +8272,8 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="ab06a5aa-8e31-4bdb-9b13-38c58a92ec8a" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="19a3940c-c740-4699-845a-46837f99845a">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{302FEEF7-88D6-41D4-B999-EFF8511D95B1}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4173999B-2FEB-4E5B-A6C7-6E33DD5EA2F7}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -8280,5 +8281,5 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4173999B-2FEB-4E5B-A6C7-6E33DD5EA2F7}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{302FEEF7-88D6-41D4-B999-EFF8511D95B1}"/>
 </file>
</xml_diff>

<commit_message>
Rename quintiles, update extraction, add zero scenarios (not run!)
</commit_message>
<xml_diff>
--- a/legacy/vivarium_gates_lsff_by_wealth_quintile/0100_data_prep/extraction/Data Extraction Sheet.xlsx
+++ b/legacy/vivarium_gates_lsff_by_wealth_quintile/0100_data_prep/extraction/Data Extraction Sheet.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28005"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28012"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uwnetid.sharepoint.com/sites/ihme_simulation_science_team/Shared Documents/Research/LSFF/04_Concept_Model_Development/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7934BE7B-3755-4AC0-B316-CDC44E903342}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{54404D2C-A9C5-464C-AB2F-9C86216971E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" firstSheet="3" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -334,7 +334,7 @@
     <t>Assumption: labeled as fortified = fortified (basically true for salt). Divided "consumed food labeled as fortified" by "consumed food".</t>
   </si>
   <si>
-    <t>Maggi cubes (most popular brand and format) claim to have 15% NRV per serving (https://www.nestle-cwa.com/en/ask-nestle/products-brands/what-is-in-the-maggi-cube), but according to Jonathan Gorstein email on July 27th it is actually 12%</t>
+    <t>Maggi cubes (most popular brand and format) claim to have 15% NRV per serving (https://www.nestle-cwa.com/en/ask-nestle/products-brands/what-is-in-the-maggi-cube), but according to Jonathan Gorstein email on July 27th it is actually 12%; https://www.wolframalpha.com/input?i=12%25+of+14mg+per+4+grams+in+mcg%2Fg</t>
   </si>
   <si>
     <t>There is some information on fraction labeled as fortified in NFCMS Table 169, but it Figure 71 shows that 95% of WRA have RBC folate insufficiency. Also: '61 percent of the non-pregnant women from households consumed bouillons that are labelled as fortified with iodine and/or iron.' There is some evidence that the rich have more bouillon labeled as fortified (Table 169).</t>
@@ -657,10 +657,10 @@
     <t>Same across all vehicles/countries/fortificants</t>
   </si>
   <si>
-    <t>15% Codex (2100mcg) per 2.5 grams; I think the 2.5 grams might be in error</t>
-  </si>
-  <si>
-    <t>15% Codex (60mcg) per 2.5 grams; I think the 2.5 grams might be in error</t>
+    <t>15% Nigeria-specific NRV per 2.5 grams; https://www.wolframalpha.com/input?i=15%25+of+22mg+per+2.5+grams+in+mcg%2Fg</t>
+  </si>
+  <si>
+    <t>15% Codex (60mcg) per 2.5 grams; https://www.wolframalpha.com/input?i=15%25+of+400mcg+per+2.5+grams+in+mcg%2Fg</t>
   </si>
   <si>
     <t>25% Codex (100mcg) per 7.1 grams</t>
@@ -871,7 +871,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -921,6 +921,9 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1418,35 +1421,35 @@
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="32" t="s">
+      <c r="B1" s="33" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="32"/>
-      <c r="D1" s="32" t="s">
+      <c r="C1" s="33"/>
+      <c r="D1" s="33" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="32"/>
-      <c r="F1" s="32" t="s">
+      <c r="E1" s="33"/>
+      <c r="F1" s="33" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="32"/>
+      <c r="G1" s="33"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="32" t="s">
+      <c r="B2" s="33" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="32"/>
-      <c r="D2" s="32" t="s">
+      <c r="C2" s="33"/>
+      <c r="D2" s="33" t="s">
         <v>6</v>
       </c>
-      <c r="E2" s="32"/>
-      <c r="F2" s="32" t="s">
+      <c r="E2" s="33"/>
+      <c r="F2" s="33" t="s">
         <v>7</v>
       </c>
-      <c r="G2" s="32"/>
+      <c r="G2" s="33"/>
     </row>
     <row r="3" spans="1:7">
       <c r="A3" s="3" t="s">
@@ -1649,44 +1652,44 @@
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="32" t="s">
+      <c r="B1" s="33" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="32"/>
-      <c r="D1" s="32" t="s">
+      <c r="C1" s="33"/>
+      <c r="D1" s="33" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="32"/>
-      <c r="F1" s="32" t="s">
+      <c r="E1" s="33"/>
+      <c r="F1" s="33" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="32"/>
+      <c r="G1" s="33"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="32" t="s">
+      <c r="B2" s="33" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="32"/>
-      <c r="D2" s="32" t="s">
+      <c r="C2" s="33"/>
+      <c r="D2" s="33" t="s">
         <v>6</v>
       </c>
-      <c r="E2" s="32"/>
-      <c r="F2" s="32" t="s">
+      <c r="E2" s="33"/>
+      <c r="F2" s="33" t="s">
         <v>7</v>
       </c>
-      <c r="G2" s="32"/>
+      <c r="G2" s="33"/>
     </row>
     <row r="3" spans="1:7">
       <c r="A3" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="B3" s="32" t="s">
+      <c r="B3" s="33" t="s">
         <v>84</v>
       </c>
-      <c r="C3" s="32"/>
+      <c r="C3" s="33"/>
       <c r="D3" s="28" t="s">
         <v>84</v>
       </c>
@@ -2308,7 +2311,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="14" spans="1:10">
+    <row r="14" spans="1:10" ht="43.5">
       <c r="A14" t="s">
         <v>2</v>
       </c>
@@ -2334,13 +2337,13 @@
         <v>193</v>
       </c>
       <c r="I14">
-        <v>840</v>
-      </c>
-      <c r="J14" t="s">
+        <v>1320</v>
+      </c>
+      <c r="J14" s="5" t="s">
         <v>195</v>
       </c>
     </row>
-    <row r="15" spans="1:10">
+    <row r="15" spans="1:10" ht="43.5">
       <c r="A15" t="s">
         <v>2</v>
       </c>
@@ -2368,7 +2371,7 @@
       <c r="I15">
         <v>24</v>
       </c>
-      <c r="J15" t="s">
+      <c r="J15" s="5" t="s">
         <v>196</v>
       </c>
     </row>
@@ -4715,7 +4718,7 @@
         <v>49</v>
       </c>
       <c r="J60" s="17">
-        <v>0.96573208722741444</v>
+        <v>0.96573208722741399</v>
       </c>
     </row>
     <row r="61" spans="1:13">
@@ -4935,76 +4938,76 @@
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="32" t="s">
+      <c r="B1" s="33" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="32"/>
-      <c r="D1" s="32"/>
-      <c r="E1" s="32"/>
-      <c r="F1" s="32" t="s">
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="32"/>
-      <c r="H1" s="32"/>
-      <c r="I1" s="32"/>
-      <c r="J1" s="33" t="s">
+      <c r="G1" s="33"/>
+      <c r="H1" s="33"/>
+      <c r="I1" s="33"/>
+      <c r="J1" s="34" t="s">
         <v>3</v>
       </c>
-      <c r="K1" s="33"/>
-      <c r="L1" s="33"/>
-      <c r="M1" s="33"/>
+      <c r="K1" s="34"/>
+      <c r="L1" s="34"/>
+      <c r="M1" s="34"/>
     </row>
     <row r="2" spans="1:13">
       <c r="A2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="32" t="s">
+      <c r="B2" s="33" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="32"/>
-      <c r="D2" s="32"/>
-      <c r="E2" s="32"/>
-      <c r="F2" s="32" t="s">
+      <c r="C2" s="33"/>
+      <c r="D2" s="33"/>
+      <c r="E2" s="33"/>
+      <c r="F2" s="33" t="s">
         <v>6</v>
       </c>
-      <c r="G2" s="32"/>
-      <c r="H2" s="32"/>
-      <c r="I2" s="32"/>
-      <c r="J2" s="32" t="s">
+      <c r="G2" s="33"/>
+      <c r="H2" s="33"/>
+      <c r="I2" s="33"/>
+      <c r="J2" s="33" t="s">
         <v>7</v>
       </c>
-      <c r="K2" s="32"/>
-      <c r="L2" s="32"/>
-      <c r="M2" s="32"/>
+      <c r="K2" s="33"/>
+      <c r="L2" s="33"/>
+      <c r="M2" s="33"/>
     </row>
     <row r="3" spans="1:13">
       <c r="A3" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="B3" s="32" t="s">
+      <c r="B3" s="33" t="s">
         <v>84</v>
       </c>
-      <c r="C3" s="32"/>
-      <c r="D3" s="32" t="s">
+      <c r="C3" s="33"/>
+      <c r="D3" s="33" t="s">
         <v>85</v>
       </c>
-      <c r="E3" s="32"/>
-      <c r="F3" s="32" t="s">
+      <c r="E3" s="33"/>
+      <c r="F3" s="33" t="s">
         <v>84</v>
       </c>
-      <c r="G3" s="32"/>
-      <c r="H3" s="32" t="s">
+      <c r="G3" s="33"/>
+      <c r="H3" s="33" t="s">
         <v>85</v>
       </c>
-      <c r="I3" s="32"/>
-      <c r="J3" s="32" t="s">
+      <c r="I3" s="33"/>
+      <c r="J3" s="33" t="s">
         <v>84</v>
       </c>
-      <c r="K3" s="32"/>
-      <c r="L3" s="32" t="s">
+      <c r="K3" s="33"/>
+      <c r="L3" s="33" t="s">
         <v>85</v>
       </c>
-      <c r="M3" s="32"/>
+      <c r="M3" s="33"/>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="3" t="s">
@@ -5512,7 +5515,7 @@
       </c>
       <c r="L9" s="9"/>
     </row>
-    <row r="10" spans="1:12">
+    <row r="10" spans="1:12" ht="101.25">
       <c r="A10" t="s">
         <v>2</v>
       </c>
@@ -5538,9 +5541,9 @@
         <v>47</v>
       </c>
       <c r="J10" s="10">
-        <v>650</v>
-      </c>
-      <c r="L10" s="9" t="s">
+        <v>420</v>
+      </c>
+      <c r="L10" s="32" t="s">
         <v>95</v>
       </c>
     </row>
@@ -5863,18 +5866,18 @@
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="32" t="s">
+      <c r="B1" s="33" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="32"/>
-      <c r="D1" s="32" t="s">
+      <c r="C1" s="33"/>
+      <c r="D1" s="33" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="32"/>
-      <c r="F1" s="33" t="s">
+      <c r="E1" s="33"/>
+      <c r="F1" s="34" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="33"/>
+      <c r="G1" s="34"/>
       <c r="H1" s="1" t="s">
         <v>26</v>
       </c>
@@ -7591,7 +7594,7 @@
       <c r="E2" t="s">
         <v>149</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" s="5" t="s">
         <v>150</v>
       </c>
       <c r="G2" s="26">
@@ -7999,17 +8002,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="ab06a5aa-8e31-4bdb-9b13-38c58a92ec8a" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="19a3940c-c740-4699-845a-46837f99845a">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -8018,7 +8010,7 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100447C4EFE3BCDC24F9D43FB479AF7E97A" ma:contentTypeVersion="17" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="710ccc9eba0c031f4d3c8297a7da4be2">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="19a3940c-c740-4699-845a-46837f99845a" xmlns:ns3="539a68f6-d0ac-4a73-9041-e1fa437c4cee" xmlns:ns4="ab06a5aa-8e31-4bdb-9b13-38c58a92ec8a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a67399e28ae6312d8947be2cafff42c1" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="19a3940c-c740-4699-845a-46837f99845a"/>
@@ -8272,14 +8264,25 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="ab06a5aa-8e31-4bdb-9b13-38c58a92ec8a" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="19a3940c-c740-4699-845a-46837f99845a">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4173999B-2FEB-4E5B-A6C7-6E33DD5EA2F7}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{44149C33-81B0-4C8D-A8B9-4C0F99EB683B}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{44149C33-81B0-4C8D-A8B9-4C0F99EB683B}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{302FEEF7-88D6-41D4-B999-EFF8511D95B1}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{302FEEF7-88D6-41D4-B999-EFF8511D95B1}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4173999B-2FEB-4E5B-A6C7-6E33DD5EA2F7}"/>
 </file>
</xml_diff>

<commit_message>
Complete scenario update, add local psimulate
</commit_message>
<xml_diff>
--- a/legacy/vivarium_gates_lsff_by_wealth_quintile/0100_data_prep/extraction/Data Extraction Sheet.xlsx
+++ b/legacy/vivarium_gates_lsff_by_wealth_quintile/0100_data_prep/extraction/Data Extraction Sheet.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28012"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28014"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uwnetid.sharepoint.com/sites/ihme_simulation_science_team/Shared Documents/Research/LSFF/04_Concept_Model_Development/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{54404D2C-A9C5-464C-AB2F-9C86216971E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{CEE2F6E1-E1CF-4143-BFE9-DE017E788A13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" firstSheet="3" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" firstSheet="10" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Country-Vehicle Progress" sheetId="1" r:id="rId1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1558" uniqueCount="216">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1552" uniqueCount="218">
   <si>
     <t>Country</t>
   </si>
@@ -292,10 +292,7 @@
     <t>Table 169, page 220 'Percentage of Non-Pregnant Women Whose Households Consumed Bouillon (purchased, branded, and labelled as fortified) by Residence, Zone, and Wealth Quintile', using 'branded' as a proxy for fortifiable and % of households as a proxy for % of product. Values obtained by dividing percent consuming branded food by percent consuming food, which is why we don't have uncertainty. A similar thing is reported in Annex 43, page 549; 'How household obtained bouillon the last time it was obtained': 'purchased', and not by wealth quintile</t>
   </si>
   <si>
-    <t>M4N Database</t>
-  </si>
-  <si>
-    <t>"Industry consolidation" sent by Jonathan Gorstein in a spreadsheet on 7/19</t>
+    <t>51.3% "Industry consolidation" sent by Jonathan Gorstein in a spreadsheet on 7/19 according to M4N Database, but on 8/15 we agreed to consider all open-market rice unfortifiable</t>
   </si>
   <si>
     <t>Fortificant</t>
@@ -348,7 +345,10 @@
     <t>Originally in mg/100g; https://www.wolframalpha.com/input?i=4.25+mg+per+100+grams+in+micrograms+per+gram</t>
   </si>
   <si>
-    <t>Originally in mcg/100g; https://www.wolframalpha.com/input?i=4.25+mg+per+100+grams+in+micrograms+per+gram</t>
+    <t>Originally in mcg/100g; https://www.wolframalpha.com/input?i=12.5+mcg+per+100+grams+in+micrograms+per+gram</t>
+  </si>
+  <si>
+    <t>Jonathan Gorstein, 8/15</t>
   </si>
   <si>
     <t>Same as intervention, for now</t>
@@ -645,7 +645,7 @@
     <t>Vehicle fortification in intervention -- amount among fortified</t>
   </si>
   <si>
-    <t>Intervention coverage % of fortifiable and unfortified</t>
+    <t>Intervention coverage % of fortifiable</t>
   </si>
   <si>
     <t>Intervention effective % of fortified</t>
@@ -654,7 +654,7 @@
     <t>Andy Garcia email 7/26</t>
   </si>
   <si>
-    <t>Same across all vehicles/countries/fortificants</t>
+    <t>Confirmed by Jonathan Gorstein, 8/15</t>
   </si>
   <si>
     <t>15% Nigeria-specific NRV per 2.5 grams; https://www.wolframalpha.com/input?i=15%25+of+22mg+per+2.5+grams+in+mcg%2Fg</t>
@@ -673,6 +673,12 @@
   </si>
   <si>
     <t>Same as baseline, PDS rice; see county-vehicle-fort extraction</t>
+  </si>
+  <si>
+    <t>https://nyaspubs.onlinelibrary.wiley.com/doi/full/10.1111/nyas.12478</t>
+  </si>
+  <si>
+    <t>https://www.wolframalpha.com/input?i=0.13+mg%2F100g+in+mcg%2Fg</t>
   </si>
   <si>
     <t>Name</t>
@@ -936,87 +942,7 @@
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="14">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="6">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -1408,7 +1334,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G9"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
     <col min="1" max="1" width="58.28515625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12.42578125" bestFit="1" customWidth="1"/>
@@ -1629,7 +1555,7 @@
     <mergeCell ref="F2:G2"/>
   </mergeCells>
   <conditionalFormatting sqref="B5:G9">
-    <cfRule type="cellIs" dxfId="13" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="5" priority="1" operator="equal">
       <formula>"Missing"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -1640,7 +1566,7 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CB686F86-0F1B-4E3A-8BF6-0236059233BB}">
   <dimension ref="A1:G8"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
     <col min="1" max="1" width="52.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="21" bestFit="1" customWidth="1"/>
@@ -1684,23 +1610,23 @@
     </row>
     <row r="3" spans="1:7">
       <c r="A3" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="B3" s="33" t="s">
         <v>83</v>
-      </c>
-      <c r="B3" s="33" t="s">
-        <v>84</v>
       </c>
       <c r="C3" s="33"/>
       <c r="D3" s="28" t="s">
+        <v>83</v>
+      </c>
+      <c r="E3" s="28" t="s">
         <v>84</v>
       </c>
-      <c r="E3" s="28" t="s">
-        <v>85</v>
-      </c>
       <c r="F3" s="28" t="s">
+        <v>83</v>
+      </c>
+      <c r="G3" s="28" t="s">
         <v>84</v>
-      </c>
-      <c r="G3" s="28" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="4" spans="1:7">
@@ -1832,47 +1758,7 @@
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="D2:E2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F6:F8">
-    <cfRule type="cellIs" dxfId="8" priority="10" operator="equal">
-      <formula>"Missing"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F8">
-    <cfRule type="cellIs" dxfId="7" priority="9" operator="equal">
-      <formula>"Missing"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G6:G8">
-    <cfRule type="cellIs" dxfId="6" priority="7" operator="equal">
-      <formula>"Missing"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B6:B8">
-    <cfRule type="cellIs" dxfId="5" priority="6" operator="equal">
-      <formula>"Missing"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B8">
-    <cfRule type="cellIs" dxfId="4" priority="5" operator="equal">
-      <formula>"Missing"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C6:C8">
-    <cfRule type="cellIs" dxfId="3" priority="4" operator="equal">
-      <formula>"Missing"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D6:D8">
-    <cfRule type="cellIs" dxfId="2" priority="3" operator="equal">
-      <formula>"Missing"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D8">
-    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
-      <formula>"Missing"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E6:E8">
+  <conditionalFormatting sqref="B6:G8">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>"Missing"</formula>
     </cfRule>
@@ -1884,7 +1770,7 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{797B3B46-8F2E-4C67-A115-D7583B1B84DB}">
   <dimension ref="A1:J19"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
     <col min="1" max="1" width="8" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10.28515625" bestFit="1" customWidth="1"/>
@@ -1903,7 +1789,7 @@
         <v>4</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>186</v>
@@ -1935,7 +1821,7 @@
         <v>6</v>
       </c>
       <c r="C2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D2" t="s">
         <v>189</v>
@@ -1950,13 +1836,10 @@
         <v>30</v>
       </c>
       <c r="H2" t="s">
-        <v>193</v>
+        <v>99</v>
       </c>
       <c r="I2" s="7">
-        <v>0.8</v>
-      </c>
-      <c r="J2" t="s">
-        <v>194</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -1967,7 +1850,7 @@
         <v>6</v>
       </c>
       <c r="C3" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D3" t="s">
         <v>189</v>
@@ -1982,13 +1865,10 @@
         <v>30</v>
       </c>
       <c r="H3" t="s">
-        <v>193</v>
+        <v>99</v>
       </c>
       <c r="I3" s="7">
-        <v>0.8</v>
-      </c>
-      <c r="J3" t="s">
-        <v>194</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -1999,7 +1879,7 @@
         <v>5</v>
       </c>
       <c r="C4" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D4" t="s">
         <v>187</v>
@@ -2031,7 +1911,7 @@
         <v>5</v>
       </c>
       <c r="C5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D5" t="s">
         <v>188</v>
@@ -2063,7 +1943,7 @@
         <v>7</v>
       </c>
       <c r="C6" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D6" t="s">
         <v>189</v>
@@ -2095,7 +1975,7 @@
         <v>7</v>
       </c>
       <c r="C7" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D7" t="s">
         <v>189</v>
@@ -2127,7 +2007,7 @@
         <v>6</v>
       </c>
       <c r="C8" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D8" t="s">
         <v>189</v>
@@ -2142,13 +2022,10 @@
         <v>30</v>
       </c>
       <c r="H8" t="s">
-        <v>193</v>
+        <v>99</v>
       </c>
       <c r="I8" s="7">
-        <v>0.8</v>
-      </c>
-      <c r="J8" t="s">
-        <v>194</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="9" spans="1:10">
@@ -2159,7 +2036,7 @@
         <v>6</v>
       </c>
       <c r="C9" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D9" t="s">
         <v>189</v>
@@ -2174,13 +2051,10 @@
         <v>30</v>
       </c>
       <c r="H9" t="s">
-        <v>193</v>
+        <v>99</v>
       </c>
       <c r="I9" s="7">
-        <v>0.8</v>
-      </c>
-      <c r="J9" t="s">
-        <v>194</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="10" spans="1:10">
@@ -2191,7 +2065,7 @@
         <v>5</v>
       </c>
       <c r="C10" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D10" t="s">
         <v>187</v>
@@ -2206,13 +2080,10 @@
         <v>30</v>
       </c>
       <c r="H10" t="s">
-        <v>193</v>
+        <v>99</v>
       </c>
       <c r="I10" s="7">
-        <v>0.8</v>
-      </c>
-      <c r="J10" t="s">
-        <v>194</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="11" spans="1:10">
@@ -2223,7 +2094,7 @@
         <v>5</v>
       </c>
       <c r="C11" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D11" t="s">
         <v>188</v>
@@ -2238,13 +2109,10 @@
         <v>30</v>
       </c>
       <c r="H11" t="s">
-        <v>193</v>
+        <v>99</v>
       </c>
       <c r="I11" s="7">
-        <v>0.8</v>
-      </c>
-      <c r="J11" t="s">
-        <v>194</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="12" spans="1:10">
@@ -2255,7 +2123,7 @@
         <v>7</v>
       </c>
       <c r="C12" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D12" t="s">
         <v>189</v>
@@ -2274,9 +2142,6 @@
       </c>
       <c r="I12" s="7">
         <v>0.8</v>
-      </c>
-      <c r="J12" t="s">
-        <v>194</v>
       </c>
     </row>
     <row r="13" spans="1:10">
@@ -2287,7 +2152,7 @@
         <v>7</v>
       </c>
       <c r="C13" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D13" t="s">
         <v>189</v>
@@ -2306,9 +2171,6 @@
       </c>
       <c r="I13" s="7">
         <v>0.8</v>
-      </c>
-      <c r="J13" t="s">
-        <v>194</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="43.5">
@@ -2319,7 +2181,7 @@
         <v>6</v>
       </c>
       <c r="C14" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D14" t="s">
         <v>189</v>
@@ -2328,10 +2190,10 @@
         <v>190</v>
       </c>
       <c r="F14" t="s">
+        <v>91</v>
+      </c>
+      <c r="G14" t="s">
         <v>92</v>
-      </c>
-      <c r="G14" t="s">
-        <v>93</v>
       </c>
       <c r="H14" t="s">
         <v>193</v>
@@ -2351,7 +2213,7 @@
         <v>6</v>
       </c>
       <c r="C15" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D15" t="s">
         <v>189</v>
@@ -2360,10 +2222,10 @@
         <v>190</v>
       </c>
       <c r="F15" t="s">
+        <v>91</v>
+      </c>
+      <c r="G15" t="s">
         <v>92</v>
-      </c>
-      <c r="G15" t="s">
-        <v>93</v>
       </c>
       <c r="H15" t="s">
         <v>193</v>
@@ -2383,7 +2245,7 @@
         <v>5</v>
       </c>
       <c r="C16" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D16" t="s">
         <v>187</v>
@@ -2392,10 +2254,10 @@
         <v>190</v>
       </c>
       <c r="F16" t="s">
+        <v>91</v>
+      </c>
+      <c r="G16" t="s">
         <v>92</v>
-      </c>
-      <c r="G16" t="s">
-        <v>93</v>
       </c>
       <c r="H16" t="s">
         <v>193</v>
@@ -2415,7 +2277,7 @@
         <v>5</v>
       </c>
       <c r="C17" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D17" t="s">
         <v>188</v>
@@ -2424,10 +2286,10 @@
         <v>190</v>
       </c>
       <c r="F17" t="s">
+        <v>91</v>
+      </c>
+      <c r="G17" t="s">
         <v>92</v>
-      </c>
-      <c r="G17" t="s">
-        <v>93</v>
       </c>
       <c r="H17" t="s">
         <v>193</v>
@@ -2447,7 +2309,7 @@
         <v>7</v>
       </c>
       <c r="C18" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D18" t="s">
         <v>189</v>
@@ -2456,10 +2318,10 @@
         <v>190</v>
       </c>
       <c r="F18" t="s">
+        <v>91</v>
+      </c>
+      <c r="G18" t="s">
         <v>92</v>
-      </c>
-      <c r="G18" t="s">
-        <v>93</v>
       </c>
       <c r="H18" t="s">
         <v>199</v>
@@ -2471,7 +2333,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="19" spans="1:10">
+    <row r="19" spans="1:10" ht="15">
       <c r="A19" t="s">
         <v>3</v>
       </c>
@@ -2479,7 +2341,7 @@
         <v>7</v>
       </c>
       <c r="C19" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D19" t="s">
         <v>189</v>
@@ -2488,19 +2350,19 @@
         <v>190</v>
       </c>
       <c r="F19" t="s">
+        <v>91</v>
+      </c>
+      <c r="G19" t="s">
         <v>92</v>
       </c>
-      <c r="G19" t="s">
-        <v>93</v>
-      </c>
-      <c r="H19" t="s">
-        <v>199</v>
+      <c r="H19" s="6" t="s">
+        <v>201</v>
       </c>
       <c r="I19">
-        <v>0.125</v>
-      </c>
-      <c r="J19" t="s">
-        <v>200</v>
+        <v>1.3</v>
+      </c>
+      <c r="J19" s="6" t="s">
+        <v>202</v>
       </c>
     </row>
   </sheetData>
@@ -2516,6 +2378,10 @@
       <formula1>"Bouillon,Salt,Rice"</formula1>
     </dataValidation>
   </dataValidations>
+  <hyperlinks>
+    <hyperlink ref="J19" r:id="rId1" xr:uid="{8B29D165-A493-48F3-B663-85CB453EE758}"/>
+    <hyperlink ref="H19" r:id="rId2" xr:uid="{3DC1B296-F88E-408E-956F-0351AD5F515E}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
@@ -2541,7 +2407,7 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{062B00F0-B806-4CE9-A08D-6C78F3C15B86}">
   <dimension ref="A1:F4"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
     <col min="2" max="2" width="40.5703125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="10.42578125" bestFit="1" customWidth="1"/>
@@ -2550,36 +2416,36 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>21</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" ht="45">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="43.5">
       <c r="A2" t="s">
         <v>49</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="C2" s="6" t="s">
         <v>51</v>
       </c>
       <c r="D2" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="E2">
         <v>2021</v>
@@ -2587,30 +2453,30 @@
     </row>
     <row r="3" spans="1:6">
       <c r="A3" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="B3" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="B4" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="D4" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="E4" s="16" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="F4" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
     </row>
   </sheetData>
@@ -2625,7 +2491,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F7501F0-08E1-4A63-A382-F6741C91E79A}">
   <dimension ref="A1:M65"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
     <col min="1" max="1" width="8" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="18.28515625" bestFit="1" customWidth="1"/>
@@ -4849,7 +4715,7 @@
         <v>0.98377281947261663</v>
       </c>
     </row>
-    <row r="65" spans="1:13">
+    <row r="65" spans="1:13" ht="57.75">
       <c r="A65" t="s">
         <v>3</v>
       </c>
@@ -4875,13 +4741,13 @@
         <v>2024</v>
       </c>
       <c r="I65" t="s">
+        <v>47</v>
+      </c>
+      <c r="J65" s="21">
+        <v>0</v>
+      </c>
+      <c r="M65" s="5" t="s">
         <v>81</v>
-      </c>
-      <c r="J65" s="21">
-        <v>0.51300000000000001</v>
-      </c>
-      <c r="M65" t="s">
-        <v>82</v>
       </c>
     </row>
   </sheetData>
@@ -4924,7 +4790,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0EC50408-61D8-4A10-93E8-9867356C2F54}">
   <dimension ref="A1:M8"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
     <col min="1" max="1" width="52.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12.42578125" bestFit="1" customWidth="1"/>
@@ -4982,30 +4848,30 @@
     </row>
     <row r="3" spans="1:13">
       <c r="A3" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="B3" s="33" t="s">
         <v>83</v>
-      </c>
-      <c r="B3" s="33" t="s">
-        <v>84</v>
       </c>
       <c r="C3" s="33"/>
       <c r="D3" s="33" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E3" s="33"/>
       <c r="F3" s="33" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="G3" s="33"/>
       <c r="H3" s="33" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="I3" s="33"/>
       <c r="J3" s="33" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="K3" s="33"/>
       <c r="L3" s="33" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="M3" s="33"/>
     </row>
@@ -5063,25 +4929,25 @@
     </row>
     <row r="6" spans="1:13">
       <c r="A6" t="s">
+        <v>85</v>
+      </c>
+      <c r="B6" t="s">
         <v>86</v>
       </c>
-      <c r="B6" t="s">
+      <c r="C6" t="s">
+        <v>86</v>
+      </c>
+      <c r="D6" t="s">
         <v>87</v>
       </c>
-      <c r="C6" t="s">
+      <c r="E6" t="s">
         <v>87</v>
       </c>
-      <c r="D6" t="s">
-        <v>88</v>
-      </c>
-      <c r="E6" t="s">
-        <v>88</v>
-      </c>
       <c r="F6" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G6" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="H6" t="str">
         <f>IF(COUNTIFS('Country-Vehicle-Fort Extraction'!$A$2:$A$940, F$1,  'Country-Vehicle-Fort Extraction'!$B$2:$B$940, F$2,  'Country-Vehicle-Fort Extraction'!$C$2:$C$940, H$3, 'Country-Vehicle-Fort Extraction'!$D$2:$D$940, "Total",  'Country-Vehicle-Fort Extraction'!$E$2:$E$940, $A6, 'Country-Vehicle-Fort Extraction'!$J$2:$J$940, "&lt;&gt;") = 0, "Missing", "Complete")</f>
@@ -5106,25 +4972,25 @@
     </row>
     <row r="7" spans="1:13">
       <c r="A7" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B7" t="s">
+        <v>86</v>
+      </c>
+      <c r="C7" t="s">
+        <v>86</v>
+      </c>
+      <c r="D7" t="s">
         <v>87</v>
       </c>
-      <c r="C7" t="s">
+      <c r="E7" t="s">
         <v>87</v>
       </c>
-      <c r="D7" t="s">
-        <v>88</v>
-      </c>
-      <c r="E7" t="s">
-        <v>88</v>
-      </c>
       <c r="F7" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G7" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="H7" t="str">
         <f>IF(COUNTIFS('Country-Vehicle-Fort Extraction'!$A$2:$A$940, F$1,  'Country-Vehicle-Fort Extraction'!$B$2:$B$940, F$2,  'Country-Vehicle-Fort Extraction'!$C$2:$C$940, H$3, 'Country-Vehicle-Fort Extraction'!$D$2:$D$940, "Total",  'Country-Vehicle-Fort Extraction'!$E$2:$E$940, $A7, 'Country-Vehicle-Fort Extraction'!$J$2:$J$940, "&lt;&gt;") = 0, "Missing", "Complete")</f>
@@ -5139,37 +5005,37 @@
         <v>Missing</v>
       </c>
       <c r="K7" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="L7" t="str">
         <f>IF(COUNTIFS('Country-Vehicle-Fort Extraction'!$A$2:$A$940, J$1,  'Country-Vehicle-Fort Extraction'!$B$2:$B$940, J$2,  'Country-Vehicle-Fort Extraction'!$C$2:$C$940, L$3, 'Country-Vehicle-Fort Extraction'!$D$2:$D$940, "All",  'Country-Vehicle-Fort Extraction'!$E$2:$E$940, $A7, 'Country-Vehicle-Fort Extraction'!$J$2:$J$940, "&lt;&gt;") = 0, "Missing", "Complete")</f>
         <v>Missing</v>
       </c>
       <c r="M7" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="8" spans="1:13">
       <c r="A8" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B8" t="s">
+        <v>86</v>
+      </c>
+      <c r="C8" t="s">
+        <v>86</v>
+      </c>
+      <c r="D8" t="s">
         <v>87</v>
       </c>
-      <c r="C8" t="s">
+      <c r="E8" t="s">
         <v>87</v>
       </c>
-      <c r="D8" t="s">
-        <v>88</v>
-      </c>
-      <c r="E8" t="s">
-        <v>88</v>
-      </c>
       <c r="F8" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G8" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="H8" t="str">
         <f>IF(COUNTIFS('Country-Vehicle-Fort Extraction'!$A$2:$A$940, F$1,  'Country-Vehicle-Fort Extraction'!$B$2:$B$940, F$2,  'Country-Vehicle-Fort Extraction'!$C$2:$C$940, H$3, 'Country-Vehicle-Fort Extraction'!$D$2:$D$940, "Total",  'Country-Vehicle-Fort Extraction'!$E$2:$E$940, $A8, 'Country-Vehicle-Fort Extraction'!$J$2:$J$940, "&lt;&gt;") = 0, "Missing", "Complete")</f>
@@ -5184,14 +5050,14 @@
         <v>Missing</v>
       </c>
       <c r="K8" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="L8" t="str">
         <f>IF(COUNTIFS('Country-Vehicle-Fort Extraction'!$A$2:$A$940, J$1,  'Country-Vehicle-Fort Extraction'!$B$2:$B$940, J$2,  'Country-Vehicle-Fort Extraction'!$C$2:$C$940, L$3, 'Country-Vehicle-Fort Extraction'!$D$2:$D$940, "All",  'Country-Vehicle-Fort Extraction'!$E$2:$E$940, $A8, 'Country-Vehicle-Fort Extraction'!$J$2:$J$940, "&lt;&gt;") = 0, "Missing", "Complete")</f>
         <v>Missing</v>
       </c>
       <c r="M8" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
   </sheetData>
@@ -5209,13 +5075,13 @@
     <mergeCell ref="F3:G3"/>
     <mergeCell ref="H3:I3"/>
   </mergeCells>
-  <conditionalFormatting sqref="B6:M6 B7:I7 I6:M7">
-    <cfRule type="cellIs" dxfId="12" priority="7" operator="equal">
+  <conditionalFormatting sqref="B6:M6 I6:M7 B7:I7">
+    <cfRule type="cellIs" dxfId="4" priority="7" operator="equal">
       <formula>"Missing"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H8:M8">
-    <cfRule type="cellIs" dxfId="11" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="3" priority="1" operator="equal">
       <formula>"Missing"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5226,7 +5092,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC26D125-533B-4E2C-8B10-83B96EF6CBCB}">
   <dimension ref="A1:L19"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
     <col min="1" max="1" width="8" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="9.5703125" bestFit="1" customWidth="1"/>
@@ -5245,7 +5111,7 @@
         <v>4</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>10</v>
@@ -5283,13 +5149,13 @@
         <v>5</v>
       </c>
       <c r="C2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D2" t="s">
         <v>27</v>
       </c>
       <c r="E2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F2" t="s">
         <v>29</v>
@@ -5312,19 +5178,19 @@
         <v>5</v>
       </c>
       <c r="C3" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D3" t="s">
         <v>27</v>
       </c>
       <c r="E3" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F3" t="s">
+        <v>91</v>
+      </c>
+      <c r="G3" s="8" t="s">
         <v>92</v>
-      </c>
-      <c r="G3" s="8" t="s">
-        <v>93</v>
       </c>
       <c r="I3" t="s">
         <v>47</v>
@@ -5341,13 +5207,13 @@
         <v>6</v>
       </c>
       <c r="C4" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D4" t="s">
         <v>33</v>
       </c>
       <c r="E4" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F4" t="s">
         <v>29</v>
@@ -5362,7 +5228,7 @@
         <v>0.61875637104994907</v>
       </c>
       <c r="L4" s="9" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="5" spans="1:12">
@@ -5373,13 +5239,13 @@
         <v>6</v>
       </c>
       <c r="C5" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D5" t="s">
         <v>37</v>
       </c>
       <c r="E5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F5" t="s">
         <v>29</v>
@@ -5403,13 +5269,13 @@
         <v>6</v>
       </c>
       <c r="C6" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D6" t="s">
         <v>38</v>
       </c>
       <c r="E6" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F6" t="s">
         <v>29</v>
@@ -5433,13 +5299,13 @@
         <v>6</v>
       </c>
       <c r="C7" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D7" t="s">
         <v>39</v>
       </c>
       <c r="E7" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F7" t="s">
         <v>29</v>
@@ -5463,13 +5329,13 @@
         <v>6</v>
       </c>
       <c r="C8" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D8" t="s">
         <v>40</v>
       </c>
       <c r="E8" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F8" t="s">
         <v>29</v>
@@ -5493,13 +5359,13 @@
         <v>6</v>
       </c>
       <c r="C9" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D9" t="s">
         <v>41</v>
       </c>
       <c r="E9" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F9" t="s">
         <v>29</v>
@@ -5515,7 +5381,7 @@
       </c>
       <c r="L9" s="9"/>
     </row>
-    <row r="10" spans="1:12" ht="101.25">
+    <row r="10" spans="1:12" ht="101.45">
       <c r="A10" t="s">
         <v>2</v>
       </c>
@@ -5523,19 +5389,19 @@
         <v>6</v>
       </c>
       <c r="C10" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D10" t="s">
         <v>27</v>
       </c>
       <c r="E10" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F10" t="s">
+        <v>91</v>
+      </c>
+      <c r="G10" s="8" t="s">
         <v>92</v>
-      </c>
-      <c r="G10" s="8" t="s">
-        <v>93</v>
       </c>
       <c r="I10" t="s">
         <v>47</v>
@@ -5544,7 +5410,7 @@
         <v>420</v>
       </c>
       <c r="L10" s="32" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="11" spans="1:12">
@@ -5555,13 +5421,13 @@
         <v>6</v>
       </c>
       <c r="C11" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D11" t="s">
         <v>27</v>
       </c>
       <c r="E11" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F11" t="s">
         <v>29</v>
@@ -5576,7 +5442,7 @@
         <v>0</v>
       </c>
       <c r="L11" s="9" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="12" spans="1:12">
@@ -5587,19 +5453,19 @@
         <v>6</v>
       </c>
       <c r="C12" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D12" t="s">
         <v>27</v>
       </c>
       <c r="E12" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F12" t="s">
+        <v>91</v>
+      </c>
+      <c r="G12" s="8" t="s">
         <v>92</v>
-      </c>
-      <c r="G12" s="8" t="s">
-        <v>93</v>
       </c>
       <c r="I12" t="s">
         <v>47</v>
@@ -5617,31 +5483,31 @@
         <v>7</v>
       </c>
       <c r="C13" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D13" t="s">
         <v>27</v>
       </c>
       <c r="E13" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F13" t="s">
+        <v>91</v>
+      </c>
+      <c r="G13" t="s">
         <v>92</v>
       </c>
-      <c r="G13" t="s">
-        <v>93</v>
-      </c>
       <c r="I13" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="J13">
         <v>42.5</v>
       </c>
       <c r="L13" s="5" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="14" spans="1:12">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" ht="43.5">
       <c r="A14" t="s">
         <v>3</v>
       </c>
@@ -5649,28 +5515,28 @@
         <v>7</v>
       </c>
       <c r="C14" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D14" t="s">
         <v>27</v>
       </c>
       <c r="E14" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F14" t="s">
+        <v>91</v>
+      </c>
+      <c r="G14" t="s">
         <v>92</v>
       </c>
-      <c r="G14" t="s">
-        <v>93</v>
-      </c>
       <c r="I14" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="J14">
         <v>0.125</v>
       </c>
-      <c r="L14" s="9" t="s">
-        <v>99</v>
+      <c r="L14" s="32" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="15" spans="1:12">
@@ -5681,13 +5547,13 @@
         <v>6</v>
       </c>
       <c r="C15" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D15" t="s">
         <v>27</v>
       </c>
       <c r="E15" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F15" t="s">
         <v>29</v>
@@ -5695,11 +5561,14 @@
       <c r="G15" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="J15" s="7">
-        <v>0.8</v>
+      <c r="I15" t="s">
+        <v>47</v>
+      </c>
+      <c r="J15" s="20">
+        <v>0</v>
       </c>
       <c r="L15" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="16" spans="1:12">
@@ -5710,13 +5579,13 @@
         <v>6</v>
       </c>
       <c r="C16" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D16" t="s">
         <v>27</v>
       </c>
       <c r="E16" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F16" t="s">
         <v>29</v>
@@ -5724,11 +5593,14 @@
       <c r="G16" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="J16" s="7">
-        <v>0.8</v>
+      <c r="I16" t="s">
+        <v>47</v>
+      </c>
+      <c r="J16" s="20">
+        <v>0</v>
       </c>
       <c r="L16" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="17" spans="1:12">
@@ -5739,13 +5611,13 @@
         <v>7</v>
       </c>
       <c r="C17" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D17" t="s">
         <v>27</v>
       </c>
       <c r="E17" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F17" t="s">
         <v>29</v>
@@ -5768,13 +5640,13 @@
         <v>7</v>
       </c>
       <c r="C18" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D18" t="s">
         <v>27</v>
       </c>
       <c r="E18" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F18" t="s">
         <v>29</v>
@@ -5797,13 +5669,13 @@
         <v>5</v>
       </c>
       <c r="C19" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D19" t="s">
         <v>27</v>
       </c>
       <c r="E19" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F19" t="s">
         <v>29</v>
@@ -5853,7 +5725,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B8AA13D-2CC0-4240-A9BF-02BB80A27D5D}">
   <dimension ref="A1:H15"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
     <col min="1" max="1" width="52.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12.42578125" bestFit="1" customWidth="1"/>
@@ -5918,10 +5790,10 @@
         <v>101</v>
       </c>
       <c r="B4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D4" t="s">
         <v>102</v>
@@ -5999,10 +5871,10 @@
         <v>107</v>
       </c>
       <c r="B7" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C7" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D7" t="s">
         <v>102</v>
@@ -6022,10 +5894,10 @@
         <v>108</v>
       </c>
       <c r="B8" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C8" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D8" t="s">
         <v>102</v>
@@ -6045,10 +5917,10 @@
         <v>109</v>
       </c>
       <c r="B9" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C9" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D9" t="s">
         <v>102</v>
@@ -6071,10 +5943,10 @@
         <v>111</v>
       </c>
       <c r="B10" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C10" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D10" t="s">
         <v>102</v>
@@ -6099,10 +5971,10 @@
         <v>113</v>
       </c>
       <c r="B11" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C11" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D11" t="s">
         <v>102</v>
@@ -6126,10 +5998,10 @@
         <v>115</v>
       </c>
       <c r="B12" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C12" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D12" t="s">
         <v>102</v>
@@ -6149,10 +6021,10 @@
         <v>116</v>
       </c>
       <c r="B13" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C13" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D13" t="s">
         <v>102</v>
@@ -6175,10 +6047,10 @@
         <v>118</v>
       </c>
       <c r="B14" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C14" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D14" t="s">
         <v>102</v>
@@ -6229,7 +6101,7 @@
     <mergeCell ref="F1:G1"/>
   </mergeCells>
   <conditionalFormatting sqref="B4:G15">
-    <cfRule type="cellIs" dxfId="10" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
       <formula>"Missing"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6240,7 +6112,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F427D668-6E74-4989-9A76-CA42E7F92A98}">
   <dimension ref="A1:J76"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
     <col min="1" max="1" width="8" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="40.42578125" customWidth="1"/>
@@ -6281,7 +6153,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="15.75">
+    <row r="2" spans="1:10" ht="15.95">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -6593,7 +6465,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="20" spans="1:10" ht="15.75">
+    <row r="20" spans="1:10" ht="15.95">
       <c r="A20" t="s">
         <v>1</v>
       </c>
@@ -7171,7 +7043,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="57" spans="1:10" ht="45">
+    <row r="57" spans="1:10" ht="43.5">
       <c r="A57" t="s">
         <v>1</v>
       </c>
@@ -7185,7 +7057,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="58" spans="1:10" ht="15.75">
+    <row r="58" spans="1:10" ht="15.95">
       <c r="A58" t="s">
         <v>1</v>
       </c>
@@ -7199,7 +7071,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="59" spans="1:10" ht="15.75">
+    <row r="59" spans="1:10" ht="15.95">
       <c r="A59" t="s">
         <v>1</v>
       </c>
@@ -7371,7 +7243,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="74" spans="1:10" ht="30">
+    <row r="74" spans="1:10" ht="29.45">
       <c r="A74" t="s">
         <v>1</v>
       </c>
@@ -7461,7 +7333,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4E519DD-7070-48BB-9F21-242D1E473943}">
   <dimension ref="A1:E4"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
     <col min="1" max="1" width="52.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12.42578125" bestFit="1" customWidth="1"/>
@@ -7498,7 +7370,7 @@
         <v>145</v>
       </c>
       <c r="B3" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C3" t="str">
         <f>IF(COUNTIFS('Vehicle Extraction'!$A$2:$A$904, C$1,  'Vehicle Extraction'!$B$2:$B$904, $A3) = 0, "Missing", "Complete")</f>
@@ -7514,7 +7386,7 @@
         <v>146</v>
       </c>
       <c r="B4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C4" t="str">
         <f>IF(COUNTIFS('Vehicle Extraction'!$A$2:$A$904, C$1,  'Vehicle Extraction'!$B$2:$B$904, $A4) = 0, "Missing", "Complete")</f>
@@ -7527,7 +7399,7 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="B3:D4">
-    <cfRule type="cellIs" dxfId="9" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
       <formula>"Missing"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -7538,7 +7410,7 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2BE8E890-3EB7-493D-B8C3-05E861B2DBA4}">
   <dimension ref="A1:I6"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
     <col min="1" max="1" width="8" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="46.42578125" bestFit="1" customWidth="1"/>
@@ -7578,7 +7450,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="115.5">
+    <row r="2" spans="1:9" ht="101.45">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -7755,7 +7627,7 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{259F6A5D-CF80-41BD-979A-295E7564EADB}">
   <dimension ref="A1:I14"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
     <col min="1" max="1" width="56.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="32.28515625" bestFit="1" customWidth="1"/>
@@ -8002,15 +7874,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100447C4EFE3BCDC24F9D43FB479AF7E97A" ma:contentTypeVersion="17" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="710ccc9eba0c031f4d3c8297a7da4be2">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="19a3940c-c740-4699-845a-46837f99845a" xmlns:ns3="539a68f6-d0ac-4a73-9041-e1fa437c4cee" xmlns:ns4="ab06a5aa-8e31-4bdb-9b13-38c58a92ec8a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a67399e28ae6312d8947be2cafff42c1" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="19a3940c-c740-4699-845a-46837f99845a"/>
@@ -8264,7 +8127,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="ab06a5aa-8e31-4bdb-9b13-38c58a92ec8a" xsi:nil="true"/>
@@ -8275,14 +8138,23 @@
 </p:properties>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{44149C33-81B0-4C8D-A8B9-4C0F99EB683B}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{302FEEF7-88D6-41D4-B999-EFF8511D95B1}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{302FEEF7-88D6-41D4-B999-EFF8511D95B1}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4173999B-2FEB-4E5B-A6C7-6E33DD5EA2F7}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4173999B-2FEB-4E5B-A6C7-6E33DD5EA2F7}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{44149C33-81B0-4C8D-A8B9-4C0F99EB683B}"/>
 </file>
</xml_diff>